<commit_message>
Update wheat monitoring to October 5 and include Zabaykalsky soft and Nizhny Novgorod durum data
</commit_message>
<xml_diff>
--- a/3d-dark/data/monitoring-src/+2.Твердая пшеница.xlsx
+++ b/3d-dark/data/monitoring-src/+2.Твердая пшеница.xlsx
@@ -5,31 +5,31 @@
   <workbookPr codeName="ЭтаКнига"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="I:\Информационный\16- МОНИТОРИНГ\Мониторинг еженедельный 2026\!Отчеты еженедельные\16 неделя на 28.09.2026\ламинирование\для СМИ\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dmitriev.aa\Desktop\ПШЕНИЦЫ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{500BCB0A-F8AE-46AF-A109-F14B26EB77E9}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E2DE612-0F8D-417C-9FFF-6BF678E8B1A0}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="18570" windowHeight="10200" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11325" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Пшеница мягкая (Л) (5)" sheetId="12" state="hidden" r:id="rId1"/>
     <sheet name="Пшеница мягкая (Л) (3)" sheetId="14" state="hidden" r:id="rId2"/>
-    <sheet name="Пшеница твердая 28 сен" sheetId="34" r:id="rId3"/>
+    <sheet name="Пшеница твердая 5 окт" sheetId="34" r:id="rId3"/>
     <sheet name="цвет (стрелочки)" sheetId="36" state="hidden" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Пшеница мягкая (Л) (3)'!$A$5:$EG$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Пшеница мягкая (Л) (5)'!$A$5:$ER$19</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Пшеница твердая 28 сен'!$A$5:$CJ$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Пшеница твердая 5 окт'!$A$5:$DA$37</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'цвет (стрелочки)'!$A$4:$M$8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Пшеница мягкая (Л) (3)'!$4:$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Пшеница мягкая (Л) (5)'!$4:$5</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Пшеница твердая 28 сен'!$4:$5</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Пшеница твердая 5 окт'!$4:$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'цвет (стрелочки)'!$4:$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Пшеница мягкая (Л) (3)'!$A$1:$E$22</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Пшеница мягкая (Л) (5)'!$A$1:$P$24</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'Пшеница твердая 28 сен'!$A$1:$P$36</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Пшеница твердая 5 окт'!$A$1:$P$37</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'цвет (стрелочки)'!$A$1:$M$8</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="72">
   <si>
     <t xml:space="preserve">Наименование субъекта  Российской федерации </t>
   </si>
@@ -433,7 +433,10 @@
     <t>Тюменская область</t>
   </si>
   <si>
-    <t>по состоянию на 28 сентября</t>
+    <t>по состоянию на 5 октября</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Нижегородская область </t>
   </si>
 </sst>
 </file>
@@ -1305,10 +1308,22 @@
     <xf numFmtId="4" fontId="28" fillId="11" borderId="5" xfId="12" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="1" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="11" borderId="1" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1347,26 +1362,20 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="20" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1376,12 +1385,6 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="1" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="11" borderId="1" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="15">
@@ -4355,44 +4358,44 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:148" s="1" customFormat="1" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A1" s="118" t="s">
+      <c r="A1" s="122" t="s">
         <v>22</v>
       </c>
-      <c r="B1" s="118"/>
-      <c r="C1" s="118"/>
-      <c r="D1" s="118"/>
-      <c r="E1" s="118"/>
-      <c r="F1" s="118"/>
-      <c r="G1" s="118"/>
-      <c r="H1" s="118"/>
-      <c r="I1" s="118"/>
-      <c r="J1" s="118"/>
-      <c r="K1" s="118"/>
-      <c r="L1" s="118"/>
-      <c r="M1" s="118"/>
-      <c r="N1" s="118"/>
-      <c r="O1" s="118"/>
-      <c r="P1" s="118"/>
+      <c r="B1" s="122"/>
+      <c r="C1" s="122"/>
+      <c r="D1" s="122"/>
+      <c r="E1" s="122"/>
+      <c r="F1" s="122"/>
+      <c r="G1" s="122"/>
+      <c r="H1" s="122"/>
+      <c r="I1" s="122"/>
+      <c r="J1" s="122"/>
+      <c r="K1" s="122"/>
+      <c r="L1" s="122"/>
+      <c r="M1" s="122"/>
+      <c r="N1" s="122"/>
+      <c r="O1" s="122"/>
+      <c r="P1" s="122"/>
     </row>
     <row r="2" spans="1:148" s="1" customFormat="1" ht="27" x14ac:dyDescent="0.35">
-      <c r="A2" s="119" t="s">
+      <c r="A2" s="123" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="119"/>
-      <c r="C2" s="119"/>
-      <c r="D2" s="119"/>
-      <c r="E2" s="119"/>
-      <c r="F2" s="119"/>
-      <c r="G2" s="119"/>
-      <c r="H2" s="119"/>
-      <c r="I2" s="119"/>
-      <c r="J2" s="119"/>
-      <c r="K2" s="119"/>
-      <c r="L2" s="119"/>
-      <c r="M2" s="119"/>
-      <c r="N2" s="119"/>
-      <c r="O2" s="119"/>
-      <c r="P2" s="119"/>
+      <c r="B2" s="123"/>
+      <c r="C2" s="123"/>
+      <c r="D2" s="123"/>
+      <c r="E2" s="123"/>
+      <c r="F2" s="123"/>
+      <c r="G2" s="123"/>
+      <c r="H2" s="123"/>
+      <c r="I2" s="123"/>
+      <c r="J2" s="123"/>
+      <c r="K2" s="123"/>
+      <c r="L2" s="123"/>
+      <c r="M2" s="123"/>
+      <c r="N2" s="123"/>
+      <c r="O2" s="123"/>
+      <c r="P2" s="123"/>
     </row>
     <row r="3" spans="1:148" x14ac:dyDescent="0.25">
       <c r="A3" s="2"/>
@@ -4413,52 +4416,52 @@
       <c r="P3" s="7"/>
     </row>
     <row r="4" spans="1:148" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="120" t="s">
+      <c r="A4" s="124" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="120" t="s">
+      <c r="B4" s="124" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="122" t="s">
+      <c r="C4" s="126" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="124" t="s">
+      <c r="D4" s="128" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="126" t="s">
+      <c r="E4" s="130" t="s">
         <v>4</v>
       </c>
-      <c r="F4" s="127" t="s">
+      <c r="F4" s="131" t="s">
         <v>5</v>
       </c>
-      <c r="G4" s="128" t="s">
+      <c r="G4" s="132" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="128"/>
-      <c r="I4" s="128" t="s">
+      <c r="H4" s="132"/>
+      <c r="I4" s="132" t="s">
         <v>7</v>
       </c>
-      <c r="J4" s="128"/>
-      <c r="K4" s="128" t="s">
+      <c r="J4" s="132"/>
+      <c r="K4" s="132" t="s">
         <v>8</v>
       </c>
-      <c r="L4" s="128"/>
-      <c r="M4" s="129" t="s">
+      <c r="L4" s="132"/>
+      <c r="M4" s="133" t="s">
         <v>9</v>
       </c>
-      <c r="N4" s="127"/>
-      <c r="O4" s="128" t="s">
+      <c r="N4" s="131"/>
+      <c r="O4" s="132" t="s">
         <v>10</v>
       </c>
-      <c r="P4" s="128"/>
+      <c r="P4" s="132"/>
     </row>
     <row r="5" spans="1:148" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="121"/>
-      <c r="B5" s="121"/>
-      <c r="C5" s="123"/>
-      <c r="D5" s="125"/>
-      <c r="E5" s="126"/>
-      <c r="F5" s="127"/>
+      <c r="A5" s="125"/>
+      <c r="B5" s="125"/>
+      <c r="C5" s="127"/>
+      <c r="D5" s="129"/>
+      <c r="E5" s="130"/>
+      <c r="F5" s="131"/>
       <c r="G5" s="28" t="s">
         <v>11</v>
       </c>
@@ -4491,7 +4494,7 @@
       </c>
     </row>
     <row r="6" spans="1:148" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="130" t="s">
+      <c r="A6" s="121" t="s">
         <v>13</v>
       </c>
       <c r="B6" s="9">
@@ -4650,7 +4653,7 @@
       <c r="DU6" s="13"/>
     </row>
     <row r="7" spans="1:148" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="131"/>
+      <c r="A7" s="134"/>
       <c r="B7" s="15">
         <v>2018</v>
       </c>
@@ -4807,7 +4810,7 @@
       <c r="DU7" s="16"/>
     </row>
     <row r="8" spans="1:148" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="130" t="s">
+      <c r="A8" s="121" t="s">
         <v>14</v>
       </c>
       <c r="B8" s="9">
@@ -4987,7 +4990,7 @@
       <c r="ER8" s="13"/>
     </row>
     <row r="9" spans="1:148" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="117"/>
+      <c r="A9" s="120"/>
       <c r="B9" s="15">
         <v>2018</v>
       </c>
@@ -5165,7 +5168,7 @@
       <c r="ER9" s="13"/>
     </row>
     <row r="10" spans="1:148" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="116" t="s">
+      <c r="A10" s="119" t="s">
         <v>15</v>
       </c>
       <c r="B10" s="9">
@@ -5214,7 +5217,7 @@
       <c r="Q10" s="10"/>
     </row>
     <row r="11" spans="1:148" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="117"/>
+      <c r="A11" s="120"/>
       <c r="B11" s="15">
         <v>2018</v>
       </c>
@@ -5265,7 +5268,7 @@
       <c r="U11" s="8"/>
     </row>
     <row r="12" spans="1:148" s="19" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="116" t="s">
+      <c r="A12" s="119" t="s">
         <v>16</v>
       </c>
       <c r="B12" s="9">
@@ -5318,7 +5321,7 @@
       <c r="U12" s="8"/>
     </row>
     <row r="13" spans="1:148" s="19" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="117"/>
+      <c r="A13" s="120"/>
       <c r="B13" s="15">
         <v>2018</v>
       </c>
@@ -5369,7 +5372,7 @@
       <c r="U13" s="8"/>
     </row>
     <row r="14" spans="1:148" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="116" t="s">
+      <c r="A14" s="119" t="s">
         <v>17</v>
       </c>
       <c r="B14" s="9">
@@ -5418,7 +5421,7 @@
       <c r="Q14" s="10"/>
     </row>
     <row r="15" spans="1:148" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="117"/>
+      <c r="A15" s="120"/>
       <c r="B15" s="15">
         <v>2018</v>
       </c>
@@ -5464,7 +5467,7 @@
       <c r="Q15" s="10"/>
     </row>
     <row r="16" spans="1:148" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="130" t="s">
+      <c r="A16" s="121" t="s">
         <v>18</v>
       </c>
       <c r="B16" s="9">
@@ -5515,7 +5518,7 @@
       <c r="Q16" s="10"/>
     </row>
     <row r="17" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="117"/>
+      <c r="A17" s="120"/>
       <c r="B17" s="15">
         <v>2018</v>
       </c>
@@ -5564,7 +5567,7 @@
       <c r="Q17" s="10"/>
     </row>
     <row r="18" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="116" t="s">
+      <c r="A18" s="119" t="s">
         <v>19</v>
       </c>
       <c r="B18" s="9">
@@ -5615,7 +5618,7 @@
       <c r="Q18" s="10"/>
     </row>
     <row r="19" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="117"/>
+      <c r="A19" s="120"/>
       <c r="B19" s="15">
         <v>2018</v>
       </c>
@@ -5683,20 +5686,20 @@
       <c r="Q20" s="10"/>
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A21" s="132" t="s">
+      <c r="A21" s="118" t="s">
         <v>26</v>
       </c>
-      <c r="B21" s="132"/>
-      <c r="C21" s="132"/>
-      <c r="D21" s="132"/>
-      <c r="E21" s="132"/>
-      <c r="F21" s="132"/>
-      <c r="G21" s="132"/>
-      <c r="H21" s="132"/>
-      <c r="I21" s="132"/>
-      <c r="J21" s="132"/>
-      <c r="K21" s="132"/>
-      <c r="L21" s="132"/>
+      <c r="B21" s="118"/>
+      <c r="C21" s="118"/>
+      <c r="D21" s="118"/>
+      <c r="E21" s="118"/>
+      <c r="F21" s="118"/>
+      <c r="G21" s="118"/>
+      <c r="H21" s="118"/>
+      <c r="I21" s="118"/>
+      <c r="J21" s="118"/>
+      <c r="K21" s="118"/>
+      <c r="L21" s="118"/>
       <c r="M21" s="27"/>
       <c r="N21" s="20" t="s">
         <v>23</v>
@@ -5709,66 +5712,66 @@
       </c>
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A22" s="132" t="s">
+      <c r="A22" s="118" t="s">
         <v>20</v>
       </c>
-      <c r="B22" s="132"/>
-      <c r="C22" s="132"/>
-      <c r="D22" s="132"/>
-      <c r="E22" s="132"/>
-      <c r="F22" s="132"/>
-      <c r="G22" s="132"/>
-      <c r="H22" s="132"/>
-      <c r="I22" s="132"/>
-      <c r="J22" s="132"/>
-      <c r="K22" s="132"/>
-      <c r="L22" s="132"/>
-      <c r="M22" s="132"/>
-      <c r="N22" s="132"/>
-      <c r="O22" s="132"/>
-      <c r="P22" s="132"/>
+      <c r="B22" s="118"/>
+      <c r="C22" s="118"/>
+      <c r="D22" s="118"/>
+      <c r="E22" s="118"/>
+      <c r="F22" s="118"/>
+      <c r="G22" s="118"/>
+      <c r="H22" s="118"/>
+      <c r="I22" s="118"/>
+      <c r="J22" s="118"/>
+      <c r="K22" s="118"/>
+      <c r="L22" s="118"/>
+      <c r="M22" s="118"/>
+      <c r="N22" s="118"/>
+      <c r="O22" s="118"/>
+      <c r="P22" s="118"/>
       <c r="Q22" s="23"/>
       <c r="R22" s="24"/>
     </row>
     <row r="23" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A23" s="132" t="s">
+      <c r="A23" s="118" t="s">
         <v>27</v>
       </c>
-      <c r="B23" s="132"/>
-      <c r="C23" s="132"/>
-      <c r="D23" s="132"/>
-      <c r="E23" s="132"/>
-      <c r="F23" s="132"/>
-      <c r="G23" s="132"/>
-      <c r="H23" s="132"/>
-      <c r="I23" s="132"/>
-      <c r="J23" s="132"/>
-      <c r="K23" s="132"/>
-      <c r="L23" s="132"/>
-      <c r="M23" s="132"/>
-      <c r="N23" s="132"/>
+      <c r="B23" s="118"/>
+      <c r="C23" s="118"/>
+      <c r="D23" s="118"/>
+      <c r="E23" s="118"/>
+      <c r="F23" s="118"/>
+      <c r="G23" s="118"/>
+      <c r="H23" s="118"/>
+      <c r="I23" s="118"/>
+      <c r="J23" s="118"/>
+      <c r="K23" s="118"/>
+      <c r="L23" s="118"/>
+      <c r="M23" s="118"/>
+      <c r="N23" s="118"/>
       <c r="O23" s="30"/>
       <c r="P23" s="30"/>
       <c r="Q23" s="23"/>
       <c r="R23" s="24"/>
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A24" s="132" t="s">
+      <c r="A24" s="118" t="s">
         <v>28</v>
       </c>
-      <c r="B24" s="132"/>
-      <c r="C24" s="132"/>
-      <c r="D24" s="132"/>
-      <c r="E24" s="132"/>
-      <c r="F24" s="132"/>
-      <c r="G24" s="132"/>
-      <c r="H24" s="132"/>
-      <c r="I24" s="132"/>
-      <c r="J24" s="132"/>
-      <c r="K24" s="132"/>
-      <c r="L24" s="132"/>
-      <c r="M24" s="132"/>
-      <c r="N24" s="132"/>
+      <c r="B24" s="118"/>
+      <c r="C24" s="118"/>
+      <c r="D24" s="118"/>
+      <c r="E24" s="118"/>
+      <c r="F24" s="118"/>
+      <c r="G24" s="118"/>
+      <c r="H24" s="118"/>
+      <c r="I24" s="118"/>
+      <c r="J24" s="118"/>
+      <c r="K24" s="118"/>
+      <c r="L24" s="118"/>
+      <c r="M24" s="118"/>
+      <c r="N24" s="118"/>
       <c r="O24"/>
       <c r="P24"/>
     </row>
@@ -23162,14 +23165,6 @@
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="A23:N23"/>
-    <mergeCell ref="A24:N24"/>
-    <mergeCell ref="A12:A13"/>
-    <mergeCell ref="A14:A15"/>
-    <mergeCell ref="A16:A17"/>
-    <mergeCell ref="A18:A19"/>
-    <mergeCell ref="A21:L21"/>
-    <mergeCell ref="A22:P22"/>
     <mergeCell ref="A10:A11"/>
     <mergeCell ref="A1:P1"/>
     <mergeCell ref="A2:P2"/>
@@ -23186,6 +23181,14 @@
     <mergeCell ref="O4:P4"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="A8:A9"/>
+    <mergeCell ref="A23:N23"/>
+    <mergeCell ref="A24:N24"/>
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="A16:A17"/>
+    <mergeCell ref="A18:A19"/>
+    <mergeCell ref="A21:L21"/>
+    <mergeCell ref="A22:P22"/>
   </mergeCells>
   <conditionalFormatting sqref="H6">
     <cfRule type="expression" dxfId="158" priority="137">
@@ -23770,18 +23773,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:137" s="1" customFormat="1" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="133"/>
-      <c r="B1" s="133"/>
-      <c r="C1" s="133"/>
-      <c r="D1" s="133"/>
-      <c r="E1" s="133"/>
+      <c r="A1" s="135"/>
+      <c r="B1" s="135"/>
+      <c r="C1" s="135"/>
+      <c r="D1" s="135"/>
+      <c r="E1" s="135"/>
     </row>
     <row r="2" spans="1:137" s="1" customFormat="1" ht="22.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="118"/>
-      <c r="B2" s="118"/>
-      <c r="C2" s="118"/>
-      <c r="D2" s="118"/>
-      <c r="E2" s="118"/>
+      <c r="A2" s="122"/>
+      <c r="B2" s="122"/>
+      <c r="C2" s="122"/>
+      <c r="D2" s="122"/>
+      <c r="E2" s="122"/>
     </row>
     <row r="3" spans="1:137" x14ac:dyDescent="0.25">
       <c r="A3" s="2"/>
@@ -31633,7 +31636,7 @@
   <sheetPr codeName="Лист6">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:CJ932"/>
+  <dimension ref="A1:DA931"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="47" style="76" bestFit="1" customWidth="1"/>
@@ -31653,43 +31656,43 @@
     <col min="17" max="16384" width="9.140625" style="73"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:88" s="71" customFormat="1" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="135" t="s">
+    <row r="1" spans="1:105" s="71" customFormat="1" ht="21" x14ac:dyDescent="0.35">
+      <c r="A1" s="136" t="s">
         <v>63</v>
       </c>
-      <c r="B1" s="135"/>
-      <c r="C1" s="135"/>
-      <c r="D1" s="135"/>
-      <c r="E1" s="135"/>
-      <c r="F1" s="135"/>
-      <c r="G1" s="135"/>
-      <c r="H1" s="135"/>
-      <c r="I1" s="135"/>
-      <c r="J1" s="135"/>
-      <c r="K1" s="135"/>
-      <c r="L1" s="135"/>
-      <c r="M1" s="135"/>
-      <c r="N1" s="135"/>
-    </row>
-    <row r="2" spans="1:88" s="71" customFormat="1" ht="21" x14ac:dyDescent="0.35">
-      <c r="A2" s="136" t="s">
+      <c r="B1" s="136"/>
+      <c r="C1" s="136"/>
+      <c r="D1" s="136"/>
+      <c r="E1" s="136"/>
+      <c r="F1" s="136"/>
+      <c r="G1" s="136"/>
+      <c r="H1" s="136"/>
+      <c r="I1" s="136"/>
+      <c r="J1" s="136"/>
+      <c r="K1" s="136"/>
+      <c r="L1" s="136"/>
+      <c r="M1" s="136"/>
+      <c r="N1" s="136"/>
+    </row>
+    <row r="2" spans="1:105" s="71" customFormat="1" ht="21" x14ac:dyDescent="0.35">
+      <c r="A2" s="137" t="s">
         <v>70</v>
       </c>
-      <c r="B2" s="136"/>
-      <c r="C2" s="136"/>
-      <c r="D2" s="136"/>
-      <c r="E2" s="136"/>
-      <c r="F2" s="136"/>
-      <c r="G2" s="136"/>
-      <c r="H2" s="136"/>
-      <c r="I2" s="136"/>
-      <c r="J2" s="136"/>
-      <c r="K2" s="136"/>
-      <c r="L2" s="136"/>
-      <c r="M2" s="136"/>
-      <c r="N2" s="136"/>
-    </row>
-    <row r="3" spans="1:88" ht="9" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="137"/>
+      <c r="C2" s="137"/>
+      <c r="D2" s="137"/>
+      <c r="E2" s="137"/>
+      <c r="F2" s="137"/>
+      <c r="G2" s="137"/>
+      <c r="H2" s="137"/>
+      <c r="I2" s="137"/>
+      <c r="J2" s="137"/>
+      <c r="K2" s="137"/>
+      <c r="L2" s="137"/>
+      <c r="M2" s="137"/>
+      <c r="N2" s="137"/>
+    </row>
+    <row r="3" spans="1:105" ht="9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="104"/>
       <c r="B3" s="104"/>
       <c r="C3" s="104"/>
@@ -31705,45 +31708,45 @@
       <c r="M3" s="104"/>
       <c r="N3" s="104"/>
     </row>
-    <row r="4" spans="1:88" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="134" t="s">
+    <row r="4" spans="1:105" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="138" t="s">
         <v>38</v>
       </c>
-      <c r="B4" s="137" t="s">
+      <c r="B4" s="139" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="134" t="s">
+      <c r="C4" s="138" t="s">
         <v>36</v>
       </c>
-      <c r="D4" s="134"/>
-      <c r="E4" s="134" t="s">
+      <c r="D4" s="138"/>
+      <c r="E4" s="138" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="134"/>
-      <c r="G4" s="134" t="s">
+      <c r="F4" s="138"/>
+      <c r="G4" s="138" t="s">
         <v>7</v>
       </c>
-      <c r="H4" s="134"/>
-      <c r="I4" s="134" t="s">
+      <c r="H4" s="138"/>
+      <c r="I4" s="138" t="s">
         <v>8</v>
       </c>
-      <c r="J4" s="134"/>
-      <c r="K4" s="134" t="s">
+      <c r="J4" s="138"/>
+      <c r="K4" s="138" t="s">
         <v>37</v>
       </c>
-      <c r="L4" s="134"/>
-      <c r="M4" s="134" t="s">
+      <c r="L4" s="138"/>
+      <c r="M4" s="138" t="s">
         <v>9</v>
       </c>
-      <c r="N4" s="134"/>
-      <c r="O4" s="134" t="s">
+      <c r="N4" s="138"/>
+      <c r="O4" s="138" t="s">
         <v>44</v>
       </c>
-      <c r="P4" s="134"/>
-    </row>
-    <row r="5" spans="1:88" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="134"/>
-      <c r="B5" s="137"/>
+      <c r="P4" s="138"/>
+    </row>
+    <row r="5" spans="1:105" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="138"/>
+      <c r="B5" s="139"/>
       <c r="C5" s="114" t="s">
         <v>11</v>
       </c>
@@ -31787,12 +31790,12 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:88" s="77" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="141" t="s">
+    <row r="6" spans="1:105" s="77" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="117" t="s">
         <v>13</v>
       </c>
       <c r="B6" s="107">
-        <v>1438.9290139999998</v>
+        <v>1522.950726</v>
       </c>
       <c r="C6" s="108">
         <v>0</v>
@@ -31804,39 +31807,37 @@
         <v>2.39127</v>
       </c>
       <c r="F6" s="108">
-        <v>0.23991233431321221</v>
+        <v>0.20841670785337121</v>
       </c>
       <c r="G6" s="107">
-        <v>236.423564</v>
+        <v>259.90216400000003</v>
       </c>
       <c r="H6" s="107">
-        <v>23.720001976309295</v>
+        <v>22.652378604192329</v>
       </c>
       <c r="I6" s="107">
-        <v>660.70211999999992</v>
+        <v>779.23487499999999</v>
       </c>
       <c r="J6" s="107">
-        <v>66.287197972160413</v>
+        <v>67.91603093420369</v>
       </c>
       <c r="K6" s="107">
-        <f>I6+G6+E6+C6</f>
-        <v>899.51695399999983</v>
+        <v>1041.528309</v>
       </c>
       <c r="L6" s="107">
-        <f>F6+D6+H6+J6</f>
-        <v>90.247112282782922</v>
+        <v>90.776826246249385</v>
       </c>
       <c r="M6" s="107">
-        <v>97.049623999999994</v>
+        <v>105.66212400000001</v>
       </c>
       <c r="N6" s="107">
-        <v>9.736835170457347</v>
+        <v>9.2092285809944876</v>
       </c>
       <c r="O6" s="107">
         <v>0.16</v>
       </c>
       <c r="P6" s="115">
-        <v>1.6052546759719295E-2</v>
+        <v>1.3945172756125154E-2</v>
       </c>
       <c r="Q6" s="76"/>
       <c r="R6" s="76"/>
@@ -31910,13 +31911,30 @@
       <c r="CH6" s="76"/>
       <c r="CI6" s="76"/>
       <c r="CJ6" s="76"/>
-    </row>
-    <row r="7" spans="1:88" s="79" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="141" t="s">
+      <c r="CK6" s="76"/>
+      <c r="CL6" s="76"/>
+      <c r="CM6" s="76"/>
+      <c r="CN6" s="76"/>
+      <c r="CO6" s="76"/>
+      <c r="CP6" s="76"/>
+      <c r="CQ6" s="76"/>
+      <c r="CR6" s="76"/>
+      <c r="CS6" s="76"/>
+      <c r="CT6" s="76"/>
+      <c r="CU6" s="76"/>
+      <c r="CV6" s="76"/>
+      <c r="CW6" s="76"/>
+      <c r="CX6" s="76"/>
+      <c r="CY6" s="76"/>
+      <c r="CZ6" s="76"/>
+      <c r="DA6" s="76"/>
+    </row>
+    <row r="7" spans="1:105" s="79" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="117" t="s">
         <v>14</v>
       </c>
       <c r="B7" s="107">
-        <v>254.040719</v>
+        <v>299.43596900000006</v>
       </c>
       <c r="C7" s="109">
         <v>0</v>
@@ -31934,27 +31952,25 @@
         <v>49.392344000000008</v>
       </c>
       <c r="H7" s="107">
-        <v>19.442687847218703</v>
+        <v>16.495127210318547</v>
       </c>
       <c r="I7" s="107">
-        <v>178.83263099999999</v>
+        <v>223.58788099999998</v>
       </c>
       <c r="J7" s="107">
-        <v>70.395262501205565</v>
+        <v>74.669680381651133</v>
       </c>
       <c r="K7" s="107">
-        <f t="shared" ref="K7:K36" si="0">I7+G7+E7+C7</f>
-        <v>228.224975</v>
+        <v>272.98022500000002</v>
       </c>
       <c r="L7" s="107">
-        <f t="shared" ref="L7:L36" si="1">F7+D7+H7+J7</f>
-        <v>89.837950348424272</v>
+        <v>91.164807591969677</v>
       </c>
       <c r="M7" s="107">
-        <v>25.815744000000002</v>
+        <v>26.455744000000003</v>
       </c>
       <c r="N7" s="107">
-        <v>10.162049651575741</v>
+        <v>8.8351924080303146</v>
       </c>
       <c r="O7" s="107">
         <v>0</v>
@@ -32034,13 +32050,30 @@
       <c r="CH7" s="78"/>
       <c r="CI7" s="78"/>
       <c r="CJ7" s="78"/>
-    </row>
-    <row r="8" spans="1:88" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="140" t="s">
+      <c r="CK7" s="78"/>
+      <c r="CL7" s="78"/>
+      <c r="CM7" s="78"/>
+      <c r="CN7" s="78"/>
+      <c r="CO7" s="78"/>
+      <c r="CP7" s="78"/>
+      <c r="CQ7" s="78"/>
+      <c r="CR7" s="78"/>
+      <c r="CS7" s="78"/>
+      <c r="CT7" s="78"/>
+      <c r="CU7" s="78"/>
+      <c r="CV7" s="78"/>
+      <c r="CW7" s="78"/>
+      <c r="CX7" s="78"/>
+      <c r="CY7" s="78"/>
+      <c r="CZ7" s="78"/>
+      <c r="DA7" s="78"/>
+    </row>
+    <row r="8" spans="1:105" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="116" t="s">
         <v>15</v>
       </c>
       <c r="B8" s="110">
-        <v>136.6</v>
+        <v>169.62</v>
       </c>
       <c r="C8" s="111"/>
       <c r="D8" s="111"/>
@@ -32050,44 +32083,38 @@
         <v>4.79</v>
       </c>
       <c r="H8" s="110">
-        <v>3.5065885797950225</v>
+        <v>2.823959438745431</v>
       </c>
       <c r="I8" s="112">
-        <v>130.54</v>
+        <v>162.91999999999999</v>
       </c>
       <c r="J8" s="110">
-        <v>95.563689604685209</v>
+        <v>96.049994104468809</v>
       </c>
       <c r="K8" s="110">
-        <f t="shared" si="0"/>
-        <v>135.32999999999998</v>
+        <v>167.70999999999998</v>
       </c>
       <c r="L8" s="110">
-        <f t="shared" si="1"/>
-        <v>99.07027818448023</v>
+        <v>98.873953543214228</v>
       </c>
       <c r="M8" s="110">
-        <v>1.27</v>
+        <v>1.91</v>
       </c>
       <c r="N8" s="110">
-        <v>0.92972181551976585</v>
+        <v>1.1260464567857562</v>
       </c>
       <c r="O8" s="110"/>
       <c r="P8" s="110"/>
     </row>
-    <row r="9" spans="1:88" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="140" t="s">
+    <row r="9" spans="1:105" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="116" t="s">
         <v>17</v>
       </c>
       <c r="B9" s="110">
-        <v>101.87631500000001</v>
-      </c>
-      <c r="C9" s="111">
-        <v>0</v>
-      </c>
-      <c r="D9" s="111">
-        <v>0</v>
-      </c>
+        <v>114.251565</v>
+      </c>
+      <c r="C9" s="111"/>
+      <c r="D9" s="111"/>
       <c r="E9" s="111">
         <v>0</v>
       </c>
@@ -32098,27 +32125,25 @@
         <v>42.602804000000006</v>
       </c>
       <c r="H9" s="110">
-        <v>41.818163525054871</v>
+        <v>37.28859556540867</v>
       </c>
       <c r="I9" s="112">
-        <v>39.221270999999994</v>
+        <v>51.596520999999996</v>
       </c>
       <c r="J9" s="110">
-        <v>38.498910173576647</v>
+        <v>45.160450099742611</v>
       </c>
       <c r="K9" s="110">
-        <f t="shared" si="0"/>
-        <v>81.824074999999993</v>
+        <v>94.199325000000002</v>
       </c>
       <c r="L9" s="110">
-        <f t="shared" si="1"/>
-        <v>80.317073698631518</v>
+        <v>82.449045665151289</v>
       </c>
       <c r="M9" s="110">
         <v>20.052240000000001</v>
       </c>
       <c r="N9" s="110">
-        <v>19.682926301368482</v>
+        <v>17.550954334848718</v>
       </c>
       <c r="O9" s="110">
         <v>0</v>
@@ -32127,8 +32152,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:88" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="140" t="s">
+    <row r="10" spans="1:105" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="116" t="s">
         <v>57</v>
       </c>
       <c r="B10" s="110">
@@ -32151,11 +32176,9 @@
         <v>65.741904053742203</v>
       </c>
       <c r="K10" s="110">
-        <f t="shared" si="0"/>
         <v>3.97994</v>
       </c>
       <c r="L10" s="110">
-        <f t="shared" si="1"/>
         <v>92.770115451585156</v>
       </c>
       <c r="M10" s="110">
@@ -32167,8 +32190,8 @@
       <c r="O10" s="110"/>
       <c r="P10" s="110"/>
     </row>
-    <row r="11" spans="1:88" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="140" t="s">
+    <row r="11" spans="1:105" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="116" t="s">
         <v>45</v>
       </c>
       <c r="B11" s="110">
@@ -32191,11 +32214,9 @@
         <v>11.456483658347336</v>
       </c>
       <c r="K11" s="110">
-        <f t="shared" si="0"/>
         <v>1.48996</v>
       </c>
       <c r="L11" s="110">
-        <f t="shared" si="1"/>
         <v>26.262696768402975</v>
       </c>
       <c r="M11" s="110">
@@ -32207,8 +32228,8 @@
       <c r="O11" s="110"/>
       <c r="P11" s="110"/>
     </row>
-    <row r="12" spans="1:88" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="140" t="s">
+    <row r="12" spans="1:105" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="116" t="s">
         <v>16</v>
       </c>
       <c r="B12" s="110">
@@ -32239,11 +32260,9 @@
         <v>100</v>
       </c>
       <c r="K12" s="110">
-        <f t="shared" si="0"/>
         <v>5.601</v>
       </c>
       <c r="L12" s="110">
-        <f t="shared" si="1"/>
         <v>100</v>
       </c>
       <c r="M12" s="110">
@@ -32259,12 +32278,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:88" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="141" t="s">
+    <row r="13" spans="1:105" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="117" t="s">
         <v>46</v>
       </c>
       <c r="B13" s="107">
-        <v>695.08834000000002</v>
+        <v>708.90910200000008</v>
       </c>
       <c r="C13" s="109">
         <v>0</v>
@@ -32276,43 +32295,41 @@
         <v>2.39127</v>
       </c>
       <c r="F13" s="109">
-        <v>0.65284867745362507</v>
+        <v>0.54727400890736067</v>
       </c>
       <c r="G13" s="107">
-        <v>137.98782</v>
+        <v>161.46642</v>
       </c>
       <c r="H13" s="107">
-        <v>37.67251953635887</v>
+        <v>36.953742144266286</v>
       </c>
       <c r="I13" s="107">
-        <v>170.14359999999999</v>
+        <v>209.35207000000003</v>
       </c>
       <c r="J13" s="107">
-        <v>46.451477347684957</v>
+        <v>47.913011337889237</v>
       </c>
       <c r="K13" s="107">
-        <f t="shared" si="0"/>
-        <v>310.52269000000001</v>
+        <v>373.20976000000002</v>
       </c>
       <c r="L13" s="107">
-        <f t="shared" si="1"/>
-        <v>84.776845561497453</v>
+        <v>85.414027491062882</v>
       </c>
       <c r="M13" s="107">
-        <v>55.599739999999997</v>
+        <v>63.572240000000001</v>
       </c>
       <c r="N13" s="107">
-        <v>15.179472299558567</v>
+        <v>14.549354376553408</v>
       </c>
       <c r="O13" s="107">
         <v>0.16</v>
       </c>
       <c r="P13" s="115">
-        <v>4.3682138943983748E-2</v>
-      </c>
-    </row>
-    <row r="14" spans="1:88" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="140" t="s">
+        <v>3.6618132383703095E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:105" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="116" t="s">
         <v>48</v>
       </c>
       <c r="B14" s="110">
@@ -32325,30 +32342,28 @@
       <c r="G14" s="110"/>
       <c r="H14" s="110"/>
       <c r="I14" s="112">
-        <v>14.76295</v>
+        <v>30.347079999999998</v>
       </c>
       <c r="J14" s="110">
-        <v>41.688304390318841</v>
+        <v>55.91074938298808</v>
       </c>
       <c r="K14" s="110">
-        <f t="shared" si="0"/>
-        <v>14.76295</v>
+        <v>30.347079999999998</v>
       </c>
       <c r="L14" s="110">
-        <f t="shared" si="1"/>
-        <v>41.688304390318841</v>
+        <v>55.91074938298808</v>
       </c>
       <c r="M14" s="110">
-        <v>20.649740000000001</v>
+        <v>23.930640000000004</v>
       </c>
       <c r="N14" s="110">
-        <v>58.311695609681166</v>
+        <v>44.08925061701192</v>
       </c>
       <c r="O14" s="110"/>
       <c r="P14" s="110"/>
     </row>
-    <row r="15" spans="1:88" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="140" t="s">
+    <row r="15" spans="1:105" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="116" t="s">
         <v>58</v>
       </c>
       <c r="B15" s="110">
@@ -32371,11 +32386,9 @@
         <v>44.089456869009581</v>
       </c>
       <c r="K15" s="110">
-        <f t="shared" si="0"/>
         <v>12.52</v>
       </c>
       <c r="L15" s="110">
-        <f t="shared" si="1"/>
         <v>100</v>
       </c>
       <c r="M15" s="110"/>
@@ -32383,12 +32396,12 @@
       <c r="O15" s="110"/>
       <c r="P15" s="110"/>
     </row>
-    <row r="16" spans="1:88" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="140" t="s">
+    <row r="16" spans="1:105" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="116" t="s">
         <v>51</v>
       </c>
       <c r="B16" s="110">
-        <v>9.844339999999999</v>
+        <v>16.96294</v>
       </c>
       <c r="C16" s="111"/>
       <c r="D16" s="111"/>
@@ -32396,27 +32409,25 @@
         <v>2.39127</v>
       </c>
       <c r="F16" s="111">
-        <v>24.29081076029475</v>
+        <v>14.097025633528151</v>
       </c>
       <c r="G16" s="110">
-        <v>2.2898200000000002</v>
+        <v>9.4084199999999996</v>
       </c>
       <c r="H16" s="110">
-        <v>23.260269352744832</v>
+        <v>55.46455979918575</v>
       </c>
       <c r="I16" s="112">
         <v>5.1632499999999997</v>
       </c>
       <c r="J16" s="110">
-        <v>52.448919886960432</v>
+        <v>30.438414567286092</v>
       </c>
       <c r="K16" s="110">
-        <f t="shared" si="0"/>
-        <v>9.8443400000000008</v>
+        <v>16.96294</v>
       </c>
       <c r="L16" s="110">
-        <f t="shared" si="1"/>
-        <v>100.00000000000001</v>
+        <v>100</v>
       </c>
       <c r="M16" s="110"/>
       <c r="N16" s="110"/>
@@ -32424,47 +32435,45 @@
       <c r="P16" s="110"/>
     </row>
     <row r="17" spans="1:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="140" t="s">
+      <c r="A17" s="116" t="s">
         <v>64</v>
       </c>
       <c r="B17" s="110">
-        <v>78.221999999999994</v>
+        <v>81.414000000000001</v>
       </c>
       <c r="C17" s="111"/>
       <c r="D17" s="111"/>
       <c r="E17" s="111"/>
       <c r="F17" s="111"/>
       <c r="G17" s="110">
-        <v>14.417999999999999</v>
+        <v>19.518000000000001</v>
       </c>
       <c r="H17" s="110">
-        <v>40.335259921556343</v>
+        <v>46.098535324024191</v>
       </c>
       <c r="I17" s="112">
-        <v>10.997400000000001</v>
+        <v>12.49174</v>
       </c>
       <c r="J17" s="110">
-        <v>30.765916733341918</v>
+        <v>29.503582213778358</v>
       </c>
       <c r="K17" s="110">
-        <f t="shared" si="0"/>
-        <v>25.415399999999998</v>
+        <v>32.009740000000001</v>
       </c>
       <c r="L17" s="110">
-        <f t="shared" si="1"/>
-        <v>71.101176654898268</v>
+        <v>75.602117537802542</v>
       </c>
       <c r="M17" s="110">
         <v>10.33</v>
       </c>
       <c r="N17" s="110">
-        <v>28.89882334510175</v>
+        <v>24.397882462197455</v>
       </c>
       <c r="O17" s="110"/>
       <c r="P17" s="110"/>
     </row>
     <row r="18" spans="1:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="140" t="s">
+      <c r="A18" s="116" t="s">
         <v>47</v>
       </c>
       <c r="B18" s="110">
@@ -32475,40 +32484,38 @@
       <c r="E18" s="111"/>
       <c r="F18" s="111"/>
       <c r="G18" s="110">
-        <v>114.28</v>
+        <v>125.54</v>
       </c>
       <c r="H18" s="110">
-        <v>41.897638949992668</v>
+        <v>40.512456434748927</v>
       </c>
       <c r="I18" s="112">
-        <v>133.69999999999999</v>
+        <v>155.83000000000001</v>
       </c>
       <c r="J18" s="110">
-        <v>49.017451239184631</v>
+        <v>50.287207951465071</v>
       </c>
       <c r="K18" s="110">
-        <f t="shared" si="0"/>
-        <v>247.98</v>
+        <v>281.37</v>
       </c>
       <c r="L18" s="110">
-        <f t="shared" si="1"/>
-        <v>90.915090189177306</v>
+        <v>90.799664386214005</v>
       </c>
       <c r="M18" s="110">
-        <v>24.62</v>
+        <v>28.35</v>
       </c>
       <c r="N18" s="110">
-        <v>9.0262501833113369</v>
+        <v>9.1487027236349547</v>
       </c>
       <c r="O18" s="110">
         <v>0.16</v>
       </c>
       <c r="P18" s="110">
-        <v>5.865962751136531E-2</v>
+        <v>5.1632890151026199E-2</v>
       </c>
     </row>
     <row r="19" spans="1:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="141" t="s">
+      <c r="A19" s="117" t="s">
         <v>18</v>
       </c>
       <c r="B19" s="107">
@@ -32539,12 +32546,10 @@
         <v>71.393276507761399</v>
       </c>
       <c r="K19" s="107">
-        <f t="shared" si="0"/>
         <v>78.570754999999991</v>
       </c>
       <c r="L19" s="107">
-        <f t="shared" si="1"/>
-        <v>92.973993150851484</v>
+        <v>92.97399315085147</v>
       </c>
       <c r="M19" s="107">
         <v>5.9375599999999995</v>
@@ -32555,12 +32560,12 @@
       <c r="O19" s="107">
         <v>0</v>
       </c>
-      <c r="P19" s="107">
+      <c r="P19" s="115">
         <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="140" t="s">
+      <c r="A20" s="116" t="s">
         <v>59</v>
       </c>
       <c r="B20" s="110">
@@ -32579,11 +32584,9 @@
       <c r="I20" s="112"/>
       <c r="J20" s="110"/>
       <c r="K20" s="110">
-        <f t="shared" si="0"/>
         <v>0.31</v>
       </c>
       <c r="L20" s="110">
-        <f t="shared" si="1"/>
         <v>100</v>
       </c>
       <c r="M20" s="110"/>
@@ -32592,7 +32595,7 @@
       <c r="P20" s="110"/>
     </row>
     <row r="21" spans="1:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="140" t="s">
+      <c r="A21" s="116" t="s">
         <v>60</v>
       </c>
       <c r="B21" s="110">
@@ -32611,11 +32614,9 @@
         <v>100</v>
       </c>
       <c r="K21" s="110">
-        <f t="shared" si="0"/>
         <v>1.34</v>
       </c>
       <c r="L21" s="110">
-        <f t="shared" si="1"/>
         <v>100</v>
       </c>
       <c r="M21" s="110"/>
@@ -32624,7 +32625,7 @@
       <c r="P21" s="110"/>
     </row>
     <row r="22" spans="1:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="140" t="s">
+      <c r="A22" s="116" t="s">
         <v>19</v>
       </c>
       <c r="B22" s="110">
@@ -32647,12 +32648,10 @@
         <v>71.197748831846269</v>
       </c>
       <c r="K22" s="110">
-        <f t="shared" si="0"/>
         <v>76.920755</v>
       </c>
       <c r="L22" s="110">
-        <f t="shared" si="1"/>
-        <v>92.834080683393097</v>
+        <v>92.834080683393083</v>
       </c>
       <c r="M22" s="110">
         <v>5.9375599999999995</v>
@@ -32664,7 +32663,7 @@
       <c r="P22" s="110"/>
     </row>
     <row r="23" spans="1:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="141" t="s">
+      <c r="A23" s="117" t="s">
         <v>52</v>
       </c>
       <c r="B23" s="107">
@@ -32678,33 +32677,31 @@
         <v>0.21</v>
       </c>
       <c r="H23" s="107">
-        <v>0.5351234384524719</v>
+        <v>0.48325651932604952</v>
       </c>
       <c r="I23" s="107">
-        <v>35.629621999999998</v>
+        <v>39.841521999999998</v>
       </c>
       <c r="J23" s="107">
-        <v>90.791646835246851</v>
+        <v>91.68416783986774</v>
       </c>
       <c r="K23" s="107">
-        <f t="shared" si="0"/>
-        <v>35.839621999999999</v>
+        <v>40.051521999999999</v>
       </c>
       <c r="L23" s="107">
-        <f t="shared" si="1"/>
-        <v>91.326770273699324</v>
+        <v>92.167424359193788</v>
       </c>
       <c r="M23" s="107">
         <v>3.4036599999999999</v>
       </c>
       <c r="N23" s="107">
-        <v>8.6732297263006704</v>
+        <v>7.8325756408061986</v>
       </c>
       <c r="O23" s="107"/>
-      <c r="P23" s="107"/>
+      <c r="P23" s="115"/>
     </row>
     <row r="24" spans="1:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="140" t="s">
+      <c r="A24" s="116" t="s">
         <v>61</v>
       </c>
       <c r="B24" s="110">
@@ -32723,11 +32720,9 @@
         <v>100</v>
       </c>
       <c r="K24" s="110">
-        <f t="shared" si="0"/>
         <v>5.3969399999999998</v>
       </c>
       <c r="L24" s="110">
-        <f t="shared" si="1"/>
         <v>100</v>
       </c>
       <c r="M24" s="110"/>
@@ -32735,8 +32730,8 @@
       <c r="O24" s="110"/>
       <c r="P24" s="110"/>
     </row>
-    <row r="25" spans="1:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="140" t="s">
+    <row r="25" spans="1:16" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A25" s="116" t="s">
         <v>55</v>
       </c>
       <c r="B25" s="110">
@@ -32755,11 +32750,9 @@
         <v>100</v>
       </c>
       <c r="K25" s="110">
-        <f t="shared" si="0"/>
         <v>2.5619999999999998</v>
       </c>
       <c r="L25" s="110">
-        <f t="shared" si="1"/>
         <v>100</v>
       </c>
       <c r="M25" s="110"/>
@@ -32768,7 +32761,7 @@
       <c r="P25" s="110"/>
     </row>
     <row r="26" spans="1:16" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A26" s="140" t="s">
+      <c r="A26" s="116" t="s">
         <v>65</v>
       </c>
       <c r="B26" s="110">
@@ -32781,17 +32774,15 @@
       <c r="G26" s="110"/>
       <c r="H26" s="110"/>
       <c r="I26" s="112">
-        <v>0.46954000000000001</v>
+        <v>3.61632</v>
       </c>
       <c r="J26" s="110">
         <v>100</v>
       </c>
       <c r="K26" s="110">
-        <f t="shared" si="0"/>
-        <v>0.46954000000000001</v>
+        <v>3.61632</v>
       </c>
       <c r="L26" s="110">
-        <f t="shared" si="1"/>
         <v>100</v>
       </c>
       <c r="M26" s="110"/>
@@ -32800,7 +32791,7 @@
       <c r="P26" s="110"/>
     </row>
     <row r="27" spans="1:16" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A27" s="140" t="s">
+      <c r="A27" s="116" t="s">
         <v>68</v>
       </c>
       <c r="B27" s="110">
@@ -32813,30 +32804,28 @@
       <c r="G27" s="110"/>
       <c r="H27" s="110"/>
       <c r="I27" s="112">
-        <v>16.993942000000001</v>
+        <v>18.059062000000001</v>
       </c>
       <c r="J27" s="110">
-        <v>93.755531479379499</v>
+        <v>94.102107235910808</v>
       </c>
       <c r="K27" s="110">
-        <f t="shared" si="0"/>
-        <v>16.993942000000001</v>
+        <v>18.059062000000001</v>
       </c>
       <c r="L27" s="110">
-        <f t="shared" si="1"/>
-        <v>93.755531479379499</v>
+        <v>94.102107235910808</v>
       </c>
       <c r="M27" s="110">
         <v>1.1318600000000001</v>
       </c>
       <c r="N27" s="110">
-        <v>6.2444685206204946</v>
+        <v>5.8978927640891881</v>
       </c>
       <c r="O27" s="110"/>
       <c r="P27" s="110"/>
     </row>
     <row r="28" spans="1:16" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A28" s="140" t="s">
+      <c r="A28" s="116" t="s">
         <v>62</v>
       </c>
       <c r="B28" s="110">
@@ -32859,12 +32848,10 @@
         <v>79.169919006252883</v>
       </c>
       <c r="K28" s="110">
-        <f t="shared" si="0"/>
         <v>9.6427000000000014</v>
       </c>
       <c r="L28" s="110">
-        <f t="shared" si="1"/>
-        <v>80.93247723362289</v>
+        <v>80.932477233622905</v>
       </c>
       <c r="M28" s="110">
         <v>2.2717999999999998</v>
@@ -32876,7 +32863,7 @@
       <c r="P28" s="110"/>
     </row>
     <row r="29" spans="1:16" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A29" s="140" t="s">
+      <c r="A29" s="116" t="s">
         <v>67</v>
       </c>
       <c r="B29" s="110">
@@ -32895,11 +32882,9 @@
         <v>100</v>
       </c>
       <c r="K29" s="110">
-        <f t="shared" si="0"/>
         <v>0.77449999999999997</v>
       </c>
       <c r="L29" s="110">
-        <f t="shared" si="1"/>
         <v>100</v>
       </c>
       <c r="M29" s="110"/>
@@ -32908,11 +32893,11 @@
       <c r="P29" s="110"/>
     </row>
     <row r="30" spans="1:16" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A30" s="141" t="s">
+      <c r="A30" s="117" t="s">
         <v>49</v>
       </c>
       <c r="B30" s="107">
-        <v>269.95399999999995</v>
+        <v>279.89600000000002</v>
       </c>
       <c r="C30" s="109">
         <v>0</v>
@@ -32930,41 +32915,39 @@
         <v>0.61799999999999999</v>
       </c>
       <c r="H30" s="107">
-        <v>0.33400597163763968</v>
+        <v>0.30182963409940711</v>
       </c>
       <c r="I30" s="107">
-        <v>183.624312</v>
+        <v>203.34894699999998</v>
       </c>
       <c r="J30" s="107">
-        <v>99.242098294260686</v>
+        <v>99.315110465226084</v>
       </c>
       <c r="K30" s="107">
-        <f t="shared" si="0"/>
-        <v>184.242312</v>
+        <v>203.96694699999998</v>
       </c>
       <c r="L30" s="107">
-        <f t="shared" si="1"/>
-        <v>99.576104265898323</v>
+        <v>99.61694009932549</v>
       </c>
       <c r="M30" s="107">
         <v>0.78432000000000002</v>
       </c>
       <c r="N30" s="107">
-        <v>0.42389573410167242</v>
+        <v>0.38305990067450968</v>
       </c>
       <c r="O30" s="107">
         <v>0</v>
       </c>
-      <c r="P30" s="107">
+      <c r="P30" s="115">
         <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:16" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A31" s="140" t="s">
+      <c r="A31" s="116" t="s">
         <v>66</v>
       </c>
       <c r="B31" s="110">
-        <v>10.9</v>
+        <v>15.189</v>
       </c>
       <c r="C31" s="111"/>
       <c r="D31" s="111"/>
@@ -32979,11 +32962,9 @@
         <v>96.815291618343096</v>
       </c>
       <c r="K31" s="110">
-        <f t="shared" si="0"/>
         <v>8.6433420000000005</v>
       </c>
       <c r="L31" s="110">
-        <f t="shared" si="1"/>
         <v>96.815291618343096</v>
       </c>
       <c r="M31" s="110">
@@ -32996,7 +32977,7 @@
       <c r="P31" s="110"/>
     </row>
     <row r="32" spans="1:16" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A32" s="140" t="s">
+      <c r="A32" s="116" t="s">
         <v>69</v>
       </c>
       <c r="B32" s="110">
@@ -33015,11 +32996,9 @@
       <c r="I32" s="112"/>
       <c r="J32" s="110"/>
       <c r="K32" s="110">
-        <f t="shared" si="0"/>
         <v>0.61799999999999999</v>
       </c>
       <c r="L32" s="110">
-        <f t="shared" si="1"/>
         <v>100</v>
       </c>
       <c r="M32" s="110"/>
@@ -33028,11 +33007,11 @@
       <c r="P32" s="110"/>
     </row>
     <row r="33" spans="1:16" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A33" s="140" t="s">
+      <c r="A33" s="116" t="s">
         <v>50</v>
       </c>
       <c r="B33" s="110">
-        <v>258.43599999999998</v>
+        <v>264.089</v>
       </c>
       <c r="C33" s="111"/>
       <c r="D33" s="111"/>
@@ -33041,34 +33020,32 @@
       <c r="G33" s="110"/>
       <c r="H33" s="110"/>
       <c r="I33" s="112">
-        <v>174.98097000000001</v>
+        <v>194.70560499999999</v>
       </c>
       <c r="J33" s="110">
-        <v>99.715068819143184</v>
+        <v>99.743859813861391</v>
       </c>
       <c r="K33" s="110">
-        <f t="shared" si="0"/>
-        <v>174.98097000000001</v>
+        <v>194.70560499999999</v>
       </c>
       <c r="L33" s="110">
-        <f t="shared" si="1"/>
-        <v>99.715068819143184</v>
+        <v>99.743859813861391</v>
       </c>
       <c r="M33" s="110">
         <v>0.5</v>
       </c>
       <c r="N33" s="110">
-        <v>0.28493118085681884</v>
+        <v>0.25614018613861012</v>
       </c>
       <c r="O33" s="110"/>
       <c r="P33" s="110"/>
     </row>
     <row r="34" spans="1:16" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A34" s="141" t="s">
+      <c r="A34" s="117" t="s">
         <v>53</v>
       </c>
       <c r="B34" s="107">
-        <v>76.390199999999993</v>
+        <v>91.253900000000002</v>
       </c>
       <c r="C34" s="109">
         <v>0</v>
@@ -33086,41 +33063,39 @@
         <v>29.977900000000002</v>
       </c>
       <c r="H34" s="107">
-        <v>44.329480726119854</v>
+        <v>38.306645863601922</v>
       </c>
       <c r="I34" s="107">
-        <v>32.1387</v>
+        <v>42.7712</v>
       </c>
       <c r="J34" s="107">
-        <v>47.524739298368068</v>
+        <v>54.654302388135612</v>
       </c>
       <c r="K34" s="107">
-        <f t="shared" si="0"/>
-        <v>62.116600000000005</v>
+        <v>72.749099999999999</v>
       </c>
       <c r="L34" s="107">
-        <f t="shared" si="1"/>
-        <v>91.854220024487915</v>
+        <v>92.960948251737534</v>
       </c>
       <c r="M34" s="107">
         <v>5.5086000000000004</v>
       </c>
       <c r="N34" s="107">
-        <v>8.1457799755120899</v>
+        <v>7.0390517482624722</v>
       </c>
       <c r="O34" s="107">
         <v>0</v>
       </c>
-      <c r="P34" s="107">
+      <c r="P34" s="115">
         <v>0</v>
       </c>
     </row>
     <row r="35" spans="1:16" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A35" s="140" t="s">
+      <c r="A35" s="116" t="s">
         <v>56</v>
       </c>
       <c r="B35" s="110">
-        <v>26.985199999999999</v>
+        <v>41.8489</v>
       </c>
       <c r="C35" s="111">
         <v>0</v>
@@ -33138,27 +33113,25 @@
         <v>3.1278999999999999</v>
       </c>
       <c r="H35" s="110">
-        <v>12.037236580822929</v>
+        <v>8.9630548718110354</v>
       </c>
       <c r="I35" s="112">
-        <v>21.4587</v>
+        <v>30.371200000000002</v>
       </c>
       <c r="J35" s="110">
-        <v>82.580468882286837</v>
+        <v>87.029231152769384</v>
       </c>
       <c r="K35" s="110">
-        <f t="shared" si="0"/>
-        <v>24.586600000000001</v>
+        <v>33.499099999999999</v>
       </c>
       <c r="L35" s="110">
-        <f t="shared" si="1"/>
-        <v>94.617705463109772</v>
+        <v>95.992286024580409</v>
       </c>
       <c r="M35" s="110">
         <v>1.3986000000000001</v>
       </c>
       <c r="N35" s="110">
-        <v>5.38229453689023</v>
+        <v>4.0077139754195832</v>
       </c>
       <c r="O35" s="110">
         <v>0</v>
@@ -33168,7 +33141,7 @@
       </c>
     </row>
     <row r="36" spans="1:16" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A36" s="140" t="s">
+      <c r="A36" s="116" t="s">
         <v>54</v>
       </c>
       <c r="B36" s="110">
@@ -33190,27 +33163,25 @@
         <v>26.85</v>
       </c>
       <c r="H36" s="110">
-        <v>64.481268011527391</v>
+        <v>61.923431734317361</v>
       </c>
       <c r="I36" s="112">
-        <v>10.68</v>
+        <v>12.4</v>
       </c>
       <c r="J36" s="110">
-        <v>25.648414985590783</v>
+        <v>28.597785977859786</v>
       </c>
       <c r="K36" s="110">
-        <f t="shared" si="0"/>
-        <v>37.53</v>
+        <v>39.25</v>
       </c>
       <c r="L36" s="110">
-        <f t="shared" si="1"/>
-        <v>90.129682997118181</v>
+        <v>90.521217712177133</v>
       </c>
       <c r="M36" s="110">
         <v>4.1100000000000003</v>
       </c>
       <c r="N36" s="110">
-        <v>9.8703170028818477</v>
+        <v>9.4787822878228809</v>
       </c>
       <c r="O36" s="110">
         <v>0</v>
@@ -33219,21 +33190,35 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A37"/>
-      <c r="B37"/>
-      <c r="C37"/>
-      <c r="D37"/>
-      <c r="E37"/>
-      <c r="F37"/>
-      <c r="G37"/>
-      <c r="H37"/>
-      <c r="I37"/>
-      <c r="J37"/>
-      <c r="K37"/>
-      <c r="L37"/>
-      <c r="M37"/>
-      <c r="N37"/>
+    <row r="37" spans="1:16" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A37" s="116" t="s">
+        <v>71</v>
+      </c>
+      <c r="B37" s="110">
+        <v>3.5101619999999998</v>
+      </c>
+      <c r="C37" s="111"/>
+      <c r="D37" s="111"/>
+      <c r="E37" s="111"/>
+      <c r="F37" s="111"/>
+      <c r="G37" s="110"/>
+      <c r="H37" s="110"/>
+      <c r="I37" s="112"/>
+      <c r="J37" s="110"/>
+      <c r="K37" s="110">
+        <v>0</v>
+      </c>
+      <c r="L37" s="110">
+        <v>0</v>
+      </c>
+      <c r="M37" s="110">
+        <v>0.96160000000000001</v>
+      </c>
+      <c r="N37" s="110">
+        <v>100</v>
+      </c>
+      <c r="O37" s="110"/>
+      <c r="P37" s="110"/>
     </row>
     <row r="38" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A38"/>
@@ -47508,20 +47493,20 @@
       <c r="N929"/>
     </row>
     <row r="930" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A930"/>
-      <c r="B930"/>
-      <c r="C930"/>
-      <c r="D930"/>
-      <c r="E930"/>
-      <c r="F930"/>
-      <c r="G930"/>
-      <c r="H930"/>
-      <c r="I930"/>
-      <c r="J930"/>
-      <c r="K930"/>
-      <c r="L930"/>
-      <c r="M930"/>
-      <c r="N930"/>
+      <c r="A930" s="81"/>
+      <c r="B930" s="81"/>
+      <c r="C930" s="81"/>
+      <c r="D930" s="81"/>
+      <c r="E930" s="81"/>
+      <c r="F930" s="81"/>
+      <c r="G930" s="81"/>
+      <c r="H930" s="81"/>
+      <c r="I930" s="81"/>
+      <c r="J930" s="81"/>
+      <c r="K930" s="81"/>
+      <c r="L930" s="81"/>
+      <c r="M930" s="81"/>
+      <c r="N930" s="81"/>
     </row>
     <row r="931" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A931" s="81"/>
@@ -47539,25 +47524,12 @@
       <c r="M931" s="81"/>
       <c r="N931" s="81"/>
     </row>
-    <row r="932" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A932" s="81"/>
-      <c r="B932" s="81"/>
-      <c r="C932" s="81"/>
-      <c r="D932" s="81"/>
-      <c r="E932" s="81"/>
-      <c r="F932" s="81"/>
-      <c r="G932" s="81"/>
-      <c r="H932" s="81"/>
-      <c r="I932" s="81"/>
-      <c r="J932" s="81"/>
-      <c r="K932" s="81"/>
-      <c r="L932" s="81"/>
-      <c r="M932" s="81"/>
-      <c r="N932" s="81"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A5:CJ36" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
+  <autoFilter ref="A5:DA37" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
   <mergeCells count="11">
+    <mergeCell ref="O4:P4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="K4:L4"/>
     <mergeCell ref="A1:N1"/>
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A4:A5"/>
@@ -47566,9 +47538,6 @@
     <mergeCell ref="E4:F4"/>
     <mergeCell ref="G4:H4"/>
     <mergeCell ref="I4:J4"/>
-    <mergeCell ref="O4:P4"/>
-    <mergeCell ref="M4:N4"/>
-    <mergeCell ref="K4:L4"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.19685039370078741" bottom="0.19685039370078741" header="0" footer="0"/>
@@ -47602,39 +47571,39 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:122" s="71" customFormat="1" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="138" t="s">
+      <c r="A1" s="140" t="s">
         <v>42</v>
       </c>
-      <c r="B1" s="138"/>
-      <c r="C1" s="138"/>
-      <c r="D1" s="138"/>
-      <c r="E1" s="138"/>
-      <c r="F1" s="138"/>
-      <c r="G1" s="138"/>
-      <c r="H1" s="138"/>
-      <c r="I1" s="138"/>
-      <c r="J1" s="138"/>
-      <c r="K1" s="138"/>
-      <c r="L1" s="138"/>
-      <c r="M1" s="138"/>
+      <c r="B1" s="140"/>
+      <c r="C1" s="140"/>
+      <c r="D1" s="140"/>
+      <c r="E1" s="140"/>
+      <c r="F1" s="140"/>
+      <c r="G1" s="140"/>
+      <c r="H1" s="140"/>
+      <c r="I1" s="140"/>
+      <c r="J1" s="140"/>
+      <c r="K1" s="140"/>
+      <c r="L1" s="140"/>
+      <c r="M1" s="140"/>
     </row>
     <row r="2" spans="1:122" s="71" customFormat="1" ht="22.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="139" t="str">
-        <f>'Пшеница твердая 28 сен'!A2:N2</f>
-        <v>по состоянию на 28 сентября</v>
-      </c>
-      <c r="B2" s="139"/>
-      <c r="C2" s="139"/>
-      <c r="D2" s="139"/>
-      <c r="E2" s="139"/>
-      <c r="F2" s="139"/>
-      <c r="G2" s="139"/>
-      <c r="H2" s="139"/>
-      <c r="I2" s="139"/>
-      <c r="J2" s="139"/>
-      <c r="K2" s="139"/>
-      <c r="L2" s="139"/>
-      <c r="M2" s="139"/>
+      <c r="A2" s="141" t="str">
+        <f>'Пшеница твердая 5 окт'!A2:N2</f>
+        <v>по состоянию на 5 октября</v>
+      </c>
+      <c r="B2" s="141"/>
+      <c r="C2" s="141"/>
+      <c r="D2" s="141"/>
+      <c r="E2" s="141"/>
+      <c r="F2" s="141"/>
+      <c r="G2" s="141"/>
+      <c r="H2" s="141"/>
+      <c r="I2" s="141"/>
+      <c r="J2" s="141"/>
+      <c r="K2" s="141"/>
+      <c r="L2" s="141"/>
+      <c r="M2" s="141"/>
     </row>
     <row r="3" spans="1:122" x14ac:dyDescent="0.25">
       <c r="A3" s="72"/>
@@ -47652,36 +47621,36 @@
       <c r="M3" s="72"/>
     </row>
     <row r="4" spans="1:122" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="128" t="s">
+      <c r="A4" s="132" t="s">
         <v>38</v>
       </c>
-      <c r="B4" s="128" t="s">
+      <c r="B4" s="132" t="s">
         <v>36</v>
       </c>
-      <c r="C4" s="128"/>
-      <c r="D4" s="128" t="s">
+      <c r="C4" s="132"/>
+      <c r="D4" s="132" t="s">
         <v>6</v>
       </c>
-      <c r="E4" s="128"/>
-      <c r="F4" s="128" t="s">
+      <c r="E4" s="132"/>
+      <c r="F4" s="132" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="128"/>
-      <c r="H4" s="128" t="s">
+      <c r="G4" s="132"/>
+      <c r="H4" s="132" t="s">
         <v>8</v>
       </c>
-      <c r="I4" s="128"/>
-      <c r="J4" s="128" t="s">
+      <c r="I4" s="132"/>
+      <c r="J4" s="132" t="s">
         <v>37</v>
       </c>
-      <c r="K4" s="128"/>
-      <c r="L4" s="128" t="s">
+      <c r="K4" s="132"/>
+      <c r="L4" s="132" t="s">
         <v>9</v>
       </c>
-      <c r="M4" s="128"/>
+      <c r="M4" s="132"/>
     </row>
     <row r="5" spans="1:122" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="128"/>
+      <c r="A5" s="132"/>
       <c r="B5" s="90" t="s">
         <v>43</v>
       </c>
@@ -47721,56 +47690,56 @@
     </row>
     <row r="6" spans="1:122" s="77" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="94" t="str">
-        <f>'Пшеница твердая 28 сен'!A6</f>
+        <f>'Пшеница твердая 5 окт'!A6</f>
         <v>Всего</v>
       </c>
       <c r="B6" s="91" t="str">
-        <f>IF('Пшеница твердая 28 сен'!D6=0,"",'Пшеница твердая 28 сен'!D6-'Пшеница твердая 28 сен'!#REF!)</f>
+        <f>IF('Пшеница твердая 5 окт'!D6=0,"",'Пшеница твердая 5 окт'!D6-'Пшеница твердая 5 окт'!#REF!)</f>
         <v/>
       </c>
       <c r="C6" s="92">
-        <f>'Пшеница твердая 28 сен'!D6</f>
+        <f>'Пшеница твердая 5 окт'!D6</f>
         <v>0</v>
       </c>
       <c r="D6" s="97" t="e">
-        <f>IF('Пшеница твердая 28 сен'!F6=0,"",'Пшеница твердая 28 сен'!F6-'Пшеница твердая 28 сен'!#REF!)</f>
+        <f>IF('Пшеница твердая 5 окт'!F6=0,"",'Пшеница твердая 5 окт'!F6-'Пшеница твердая 5 окт'!#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="E6" s="92">
-        <f>'Пшеница твердая 28 сен'!F6</f>
-        <v>0.23991233431321221</v>
+        <f>'Пшеница твердая 5 окт'!F6</f>
+        <v>0.20841670785337121</v>
       </c>
       <c r="F6" s="97" t="e">
-        <f>IF('Пшеница твердая 28 сен'!H6=0,"",'Пшеница твердая 28 сен'!H6-'Пшеница твердая 28 сен'!#REF!)</f>
+        <f>IF('Пшеница твердая 5 окт'!H6=0,"",'Пшеница твердая 5 окт'!H6-'Пшеница твердая 5 окт'!#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="G6" s="92">
-        <f>'Пшеница твердая 28 сен'!H6</f>
-        <v>23.720001976309295</v>
+        <f>'Пшеница твердая 5 окт'!H6</f>
+        <v>22.652378604192329</v>
       </c>
       <c r="H6" s="97" t="e">
-        <f>IF('Пшеница твердая 28 сен'!J6=0,"",'Пшеница твердая 28 сен'!J6-'Пшеница твердая 28 сен'!#REF!)</f>
+        <f>IF('Пшеница твердая 5 окт'!J6=0,"",'Пшеница твердая 5 окт'!J6-'Пшеница твердая 5 окт'!#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="I6" s="92">
-        <f>'Пшеница твердая 28 сен'!J6</f>
-        <v>66.287197972160413</v>
+        <f>'Пшеница твердая 5 окт'!J6</f>
+        <v>67.91603093420369</v>
       </c>
       <c r="J6" s="97" t="e">
-        <f>IF('Пшеница твердая 28 сен'!L6=0,"",'Пшеница твердая 28 сен'!L6-'Пшеница твердая 28 сен'!#REF!)</f>
+        <f>IF('Пшеница твердая 5 окт'!L6=0,"",'Пшеница твердая 5 окт'!L6-'Пшеница твердая 5 окт'!#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="K6" s="92">
-        <f>'Пшеница твердая 28 сен'!L6</f>
-        <v>90.247112282782922</v>
+        <f>'Пшеница твердая 5 окт'!L6</f>
+        <v>90.776826246249385</v>
       </c>
       <c r="L6" s="99" t="e">
-        <f>IF('Пшеница твердая 28 сен'!N6=0,"",'Пшеница твердая 28 сен'!N6-'Пшеница твердая 28 сен'!#REF!)</f>
+        <f>IF('Пшеница твердая 5 окт'!N6=0,"",'Пшеница твердая 5 окт'!N6-'Пшеница твердая 5 окт'!#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="M6" s="92">
-        <f>'Пшеница твердая 28 сен'!N6</f>
-        <v>9.736835170457347</v>
+        <f>'Пшеница твердая 5 окт'!N6</f>
+        <v>9.2092285809944876</v>
       </c>
       <c r="N6" s="73"/>
       <c r="O6" s="73"/>
@@ -47884,56 +47853,56 @@
     </row>
     <row r="7" spans="1:122" s="79" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="95" t="str">
-        <f>'Пшеница твердая 28 сен'!A7</f>
+        <f>'Пшеница твердая 5 окт'!A7</f>
         <v>Южный фед. округ</v>
       </c>
       <c r="B7" s="101" t="str">
-        <f>IF('Пшеница твердая 28 сен'!D7=0,"",'Пшеница твердая 28 сен'!D7-'Пшеница твердая 28 сен'!#REF!)</f>
+        <f>IF('Пшеница твердая 5 окт'!D7=0,"",'Пшеница твердая 5 окт'!D7-'Пшеница твердая 5 окт'!#REF!)</f>
         <v/>
       </c>
       <c r="C7" s="93">
-        <f>'Пшеница твердая 28 сен'!D7</f>
+        <f>'Пшеница твердая 5 окт'!D7</f>
         <v>0</v>
       </c>
       <c r="D7" s="98" t="str">
-        <f>IF('Пшеница твердая 28 сен'!F7=0,"",'Пшеница твердая 28 сен'!F7-'Пшеница твердая 28 сен'!#REF!)</f>
+        <f>IF('Пшеница твердая 5 окт'!F7=0,"",'Пшеница твердая 5 окт'!F7-'Пшеница твердая 5 окт'!#REF!)</f>
         <v/>
       </c>
       <c r="E7" s="93">
-        <f>'Пшеница твердая 28 сен'!F7</f>
+        <f>'Пшеница твердая 5 окт'!F7</f>
         <v>0</v>
       </c>
       <c r="F7" s="98" t="e">
-        <f>IF('Пшеница твердая 28 сен'!H7=0,"",'Пшеница твердая 28 сен'!H7-'Пшеница твердая 28 сен'!#REF!)</f>
+        <f>IF('Пшеница твердая 5 окт'!H7=0,"",'Пшеница твердая 5 окт'!H7-'Пшеница твердая 5 окт'!#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="G7" s="93">
-        <f>'Пшеница твердая 28 сен'!H7</f>
-        <v>19.442687847218703</v>
+        <f>'Пшеница твердая 5 окт'!H7</f>
+        <v>16.495127210318547</v>
       </c>
       <c r="H7" s="98" t="e">
-        <f>IF('Пшеница твердая 28 сен'!J7=0,"",'Пшеница твердая 28 сен'!J7-'Пшеница твердая 28 сен'!#REF!)</f>
+        <f>IF('Пшеница твердая 5 окт'!J7=0,"",'Пшеница твердая 5 окт'!J7-'Пшеница твердая 5 окт'!#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="I7" s="93">
-        <f>'Пшеница твердая 28 сен'!J7</f>
-        <v>70.395262501205565</v>
+        <f>'Пшеница твердая 5 окт'!J7</f>
+        <v>74.669680381651133</v>
       </c>
       <c r="J7" s="98" t="e">
-        <f>IF('Пшеница твердая 28 сен'!L7=0,"",'Пшеница твердая 28 сен'!L7-'Пшеница твердая 28 сен'!#REF!)</f>
+        <f>IF('Пшеница твердая 5 окт'!L7=0,"",'Пшеница твердая 5 окт'!L7-'Пшеница твердая 5 окт'!#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="K7" s="93">
-        <f>'Пшеница твердая 28 сен'!L7</f>
-        <v>89.837950348424272</v>
+        <f>'Пшеница твердая 5 окт'!L7</f>
+        <v>91.164807591969677</v>
       </c>
       <c r="L7" s="100" t="e">
-        <f>IF('Пшеница твердая 28 сен'!N7=0,"",'Пшеница твердая 28 сен'!N7-'Пшеница твердая 28 сен'!#REF!)</f>
+        <f>IF('Пшеница твердая 5 окт'!N7=0,"",'Пшеница твердая 5 окт'!N7-'Пшеница твердая 5 окт'!#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="M7" s="93">
-        <f>'Пшеница твердая 28 сен'!N7</f>
-        <v>10.162049651575741</v>
+        <f>'Пшеница твердая 5 окт'!N7</f>
+        <v>8.8351924080303146</v>
       </c>
       <c r="N7" s="73"/>
       <c r="O7" s="73"/>
@@ -48047,55 +48016,55 @@
     </row>
     <row r="8" spans="1:122" s="77" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="96" t="e">
-        <f>'Пшеница твердая 28 сен'!#REF!</f>
+        <f>'Пшеница твердая 5 окт'!#REF!</f>
         <v>#REF!</v>
       </c>
       <c r="B8" s="91" t="e">
-        <f>IF('Пшеница твердая 28 сен'!#REF!=0,"",'Пшеница твердая 28 сен'!#REF!-'Пшеница твердая 28 сен'!#REF!)</f>
+        <f>IF('Пшеница твердая 5 окт'!#REF!=0,"",'Пшеница твердая 5 окт'!#REF!-'Пшеница твердая 5 окт'!#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="C8" s="92" t="e">
-        <f>'Пшеница твердая 28 сен'!#REF!</f>
+        <f>'Пшеница твердая 5 окт'!#REF!</f>
         <v>#REF!</v>
       </c>
       <c r="D8" s="91" t="e">
-        <f>IF('Пшеница твердая 28 сен'!#REF!=0,"",'Пшеница твердая 28 сен'!#REF!-'Пшеница твердая 28 сен'!#REF!)</f>
+        <f>IF('Пшеница твердая 5 окт'!#REF!=0,"",'Пшеница твердая 5 окт'!#REF!-'Пшеница твердая 5 окт'!#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="E8" s="92" t="e">
-        <f>'Пшеница твердая 28 сен'!#REF!</f>
+        <f>'Пшеница твердая 5 окт'!#REF!</f>
         <v>#REF!</v>
       </c>
       <c r="F8" s="91" t="e">
-        <f>IF('Пшеница твердая 28 сен'!#REF!=0,"",'Пшеница твердая 28 сен'!#REF!-'Пшеница твердая 28 сен'!#REF!)</f>
+        <f>IF('Пшеница твердая 5 окт'!#REF!=0,"",'Пшеница твердая 5 окт'!#REF!-'Пшеница твердая 5 окт'!#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="G8" s="92" t="e">
-        <f>'Пшеница твердая 28 сен'!#REF!</f>
+        <f>'Пшеница твердая 5 окт'!#REF!</f>
         <v>#REF!</v>
       </c>
       <c r="H8" s="91" t="e">
-        <f>IF('Пшеница твердая 28 сен'!#REF!=0,"",'Пшеница твердая 28 сен'!#REF!-'Пшеница твердая 28 сен'!#REF!)</f>
+        <f>IF('Пшеница твердая 5 окт'!#REF!=0,"",'Пшеница твердая 5 окт'!#REF!-'Пшеница твердая 5 окт'!#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="I8" s="92" t="e">
-        <f>'Пшеница твердая 28 сен'!#REF!</f>
+        <f>'Пшеница твердая 5 окт'!#REF!</f>
         <v>#REF!</v>
       </c>
       <c r="J8" s="91" t="e">
-        <f>IF('Пшеница твердая 28 сен'!#REF!=0,"",'Пшеница твердая 28 сен'!#REF!-'Пшеница твердая 28 сен'!#REF!)</f>
+        <f>IF('Пшеница твердая 5 окт'!#REF!=0,"",'Пшеница твердая 5 окт'!#REF!-'Пшеница твердая 5 окт'!#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="K8" s="92" t="e">
-        <f>'Пшеница твердая 28 сен'!#REF!</f>
+        <f>'Пшеница твердая 5 окт'!#REF!</f>
         <v>#REF!</v>
       </c>
       <c r="L8" s="91" t="e">
-        <f>IF('Пшеница твердая 28 сен'!#REF!=0,"",'Пшеница твердая 28 сен'!#REF!-'Пшеница твердая 28 сен'!#REF!)</f>
+        <f>IF('Пшеница твердая 5 окт'!#REF!=0,"",'Пшеница твердая 5 окт'!#REF!-'Пшеница твердая 5 окт'!#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="M8" s="92" t="e">
-        <f>'Пшеница твердая 28 сен'!#REF!</f>
+        <f>'Пшеница твердая 5 окт'!#REF!</f>
         <v>#REF!</v>
       </c>
       <c r="N8" s="73"/>

</xml_diff>

<commit_message>
Release full Windows 1.0.22 from main 93ef532 without checks
</commit_message>
<xml_diff>
--- a/3d-dark/data/monitoring-src/+2.Твердая пшеница.xlsx
+++ b/3d-dark/data/monitoring-src/+2.Твердая пшеница.xlsx
@@ -5,31 +5,31 @@
   <workbookPr codeName="ЭтаКнига"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="I:\Информационный\16- МОНИТОРИНГ\Мониторинг еженедельный 2026\!Отчеты еженедельные\16 неделя на 28.09.2026\ламинирование\для СМИ\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dmitriev.aa\Desktop\ПШЕНИЦЫ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{500BCB0A-F8AE-46AF-A109-F14B26EB77E9}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E2DE612-0F8D-417C-9FFF-6BF678E8B1A0}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="18570" windowHeight="10200" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11325" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Пшеница мягкая (Л) (5)" sheetId="12" state="hidden" r:id="rId1"/>
     <sheet name="Пшеница мягкая (Л) (3)" sheetId="14" state="hidden" r:id="rId2"/>
-    <sheet name="Пшеница твердая 28 сен" sheetId="34" r:id="rId3"/>
+    <sheet name="Пшеница твердая 5 окт" sheetId="34" r:id="rId3"/>
     <sheet name="цвет (стрелочки)" sheetId="36" state="hidden" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Пшеница мягкая (Л) (3)'!$A$5:$EG$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Пшеница мягкая (Л) (5)'!$A$5:$ER$19</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Пшеница твердая 28 сен'!$A$5:$CJ$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Пшеница твердая 5 окт'!$A$5:$DA$37</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'цвет (стрелочки)'!$A$4:$M$8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Пшеница мягкая (Л) (3)'!$4:$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Пшеница мягкая (Л) (5)'!$4:$5</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Пшеница твердая 28 сен'!$4:$5</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Пшеница твердая 5 окт'!$4:$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'цвет (стрелочки)'!$4:$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Пшеница мягкая (Л) (3)'!$A$1:$E$22</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Пшеница мягкая (Л) (5)'!$A$1:$P$24</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'Пшеница твердая 28 сен'!$A$1:$P$36</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Пшеница твердая 5 окт'!$A$1:$P$37</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'цвет (стрелочки)'!$A$1:$M$8</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="72">
   <si>
     <t xml:space="preserve">Наименование субъекта  Российской федерации </t>
   </si>
@@ -433,7 +433,10 @@
     <t>Тюменская область</t>
   </si>
   <si>
-    <t>по состоянию на 28 сентября</t>
+    <t>по состоянию на 5 октября</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Нижегородская область </t>
   </si>
 </sst>
 </file>
@@ -1305,10 +1308,22 @@
     <xf numFmtId="4" fontId="28" fillId="11" borderId="5" xfId="12" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="1" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="11" borderId="1" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1347,26 +1362,20 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="20" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1376,12 +1385,6 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="1" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="11" borderId="1" xfId="12" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="15">
@@ -4355,44 +4358,44 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:148" s="1" customFormat="1" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A1" s="118" t="s">
+      <c r="A1" s="122" t="s">
         <v>22</v>
       </c>
-      <c r="B1" s="118"/>
-      <c r="C1" s="118"/>
-      <c r="D1" s="118"/>
-      <c r="E1" s="118"/>
-      <c r="F1" s="118"/>
-      <c r="G1" s="118"/>
-      <c r="H1" s="118"/>
-      <c r="I1" s="118"/>
-      <c r="J1" s="118"/>
-      <c r="K1" s="118"/>
-      <c r="L1" s="118"/>
-      <c r="M1" s="118"/>
-      <c r="N1" s="118"/>
-      <c r="O1" s="118"/>
-      <c r="P1" s="118"/>
+      <c r="B1" s="122"/>
+      <c r="C1" s="122"/>
+      <c r="D1" s="122"/>
+      <c r="E1" s="122"/>
+      <c r="F1" s="122"/>
+      <c r="G1" s="122"/>
+      <c r="H1" s="122"/>
+      <c r="I1" s="122"/>
+      <c r="J1" s="122"/>
+      <c r="K1" s="122"/>
+      <c r="L1" s="122"/>
+      <c r="M1" s="122"/>
+      <c r="N1" s="122"/>
+      <c r="O1" s="122"/>
+      <c r="P1" s="122"/>
     </row>
     <row r="2" spans="1:148" s="1" customFormat="1" ht="27" x14ac:dyDescent="0.35">
-      <c r="A2" s="119" t="s">
+      <c r="A2" s="123" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="119"/>
-      <c r="C2" s="119"/>
-      <c r="D2" s="119"/>
-      <c r="E2" s="119"/>
-      <c r="F2" s="119"/>
-      <c r="G2" s="119"/>
-      <c r="H2" s="119"/>
-      <c r="I2" s="119"/>
-      <c r="J2" s="119"/>
-      <c r="K2" s="119"/>
-      <c r="L2" s="119"/>
-      <c r="M2" s="119"/>
-      <c r="N2" s="119"/>
-      <c r="O2" s="119"/>
-      <c r="P2" s="119"/>
+      <c r="B2" s="123"/>
+      <c r="C2" s="123"/>
+      <c r="D2" s="123"/>
+      <c r="E2" s="123"/>
+      <c r="F2" s="123"/>
+      <c r="G2" s="123"/>
+      <c r="H2" s="123"/>
+      <c r="I2" s="123"/>
+      <c r="J2" s="123"/>
+      <c r="K2" s="123"/>
+      <c r="L2" s="123"/>
+      <c r="M2" s="123"/>
+      <c r="N2" s="123"/>
+      <c r="O2" s="123"/>
+      <c r="P2" s="123"/>
     </row>
     <row r="3" spans="1:148" x14ac:dyDescent="0.25">
       <c r="A3" s="2"/>
@@ -4413,52 +4416,52 @@
       <c r="P3" s="7"/>
     </row>
     <row r="4" spans="1:148" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="120" t="s">
+      <c r="A4" s="124" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="120" t="s">
+      <c r="B4" s="124" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="122" t="s">
+      <c r="C4" s="126" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="124" t="s">
+      <c r="D4" s="128" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="126" t="s">
+      <c r="E4" s="130" t="s">
         <v>4</v>
       </c>
-      <c r="F4" s="127" t="s">
+      <c r="F4" s="131" t="s">
         <v>5</v>
       </c>
-      <c r="G4" s="128" t="s">
+      <c r="G4" s="132" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="128"/>
-      <c r="I4" s="128" t="s">
+      <c r="H4" s="132"/>
+      <c r="I4" s="132" t="s">
         <v>7</v>
       </c>
-      <c r="J4" s="128"/>
-      <c r="K4" s="128" t="s">
+      <c r="J4" s="132"/>
+      <c r="K4" s="132" t="s">
         <v>8</v>
       </c>
-      <c r="L4" s="128"/>
-      <c r="M4" s="129" t="s">
+      <c r="L4" s="132"/>
+      <c r="M4" s="133" t="s">
         <v>9</v>
       </c>
-      <c r="N4" s="127"/>
-      <c r="O4" s="128" t="s">
+      <c r="N4" s="131"/>
+      <c r="O4" s="132" t="s">
         <v>10</v>
       </c>
-      <c r="P4" s="128"/>
+      <c r="P4" s="132"/>
     </row>
     <row r="5" spans="1:148" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="121"/>
-      <c r="B5" s="121"/>
-      <c r="C5" s="123"/>
-      <c r="D5" s="125"/>
-      <c r="E5" s="126"/>
-      <c r="F5" s="127"/>
+      <c r="A5" s="125"/>
+      <c r="B5" s="125"/>
+      <c r="C5" s="127"/>
+      <c r="D5" s="129"/>
+      <c r="E5" s="130"/>
+      <c r="F5" s="131"/>
       <c r="G5" s="28" t="s">
         <v>11</v>
       </c>
@@ -4491,7 +4494,7 @@
       </c>
     </row>
     <row r="6" spans="1:148" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="130" t="s">
+      <c r="A6" s="121" t="s">
         <v>13</v>
       </c>
       <c r="B6" s="9">
@@ -4650,7 +4653,7 @@
       <c r="DU6" s="13"/>
     </row>
     <row r="7" spans="1:148" s="17" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="131"/>
+      <c r="A7" s="134"/>
       <c r="B7" s="15">
         <v>2018</v>
       </c>
@@ -4807,7 +4810,7 @@
       <c r="DU7" s="16"/>
     </row>
     <row r="8" spans="1:148" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="130" t="s">
+      <c r="A8" s="121" t="s">
         <v>14</v>
       </c>
       <c r="B8" s="9">
@@ -4987,7 +4990,7 @@
       <c r="ER8" s="13"/>
     </row>
     <row r="9" spans="1:148" s="14" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="117"/>
+      <c r="A9" s="120"/>
       <c r="B9" s="15">
         <v>2018</v>
       </c>
@@ -5165,7 +5168,7 @@
       <c r="ER9" s="13"/>
     </row>
     <row r="10" spans="1:148" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="116" t="s">
+      <c r="A10" s="119" t="s">
         <v>15</v>
       </c>
       <c r="B10" s="9">
@@ -5214,7 +5217,7 @@
       <c r="Q10" s="10"/>
     </row>
     <row r="11" spans="1:148" s="18" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="117"/>
+      <c r="A11" s="120"/>
       <c r="B11" s="15">
         <v>2018</v>
       </c>
@@ -5265,7 +5268,7 @@
       <c r="U11" s="8"/>
     </row>
     <row r="12" spans="1:148" s="19" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="116" t="s">
+      <c r="A12" s="119" t="s">
         <v>16</v>
       </c>
       <c r="B12" s="9">
@@ -5318,7 +5321,7 @@
       <c r="U12" s="8"/>
     </row>
     <row r="13" spans="1:148" s="19" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="117"/>
+      <c r="A13" s="120"/>
       <c r="B13" s="15">
         <v>2018</v>
       </c>
@@ -5369,7 +5372,7 @@
       <c r="U13" s="8"/>
     </row>
     <row r="14" spans="1:148" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="116" t="s">
+      <c r="A14" s="119" t="s">
         <v>17</v>
       </c>
       <c r="B14" s="9">
@@ -5418,7 +5421,7 @@
       <c r="Q14" s="10"/>
     </row>
     <row r="15" spans="1:148" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="117"/>
+      <c r="A15" s="120"/>
       <c r="B15" s="15">
         <v>2018</v>
       </c>
@@ -5464,7 +5467,7 @@
       <c r="Q15" s="10"/>
     </row>
     <row r="16" spans="1:148" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="130" t="s">
+      <c r="A16" s="121" t="s">
         <v>18</v>
       </c>
       <c r="B16" s="9">
@@ -5515,7 +5518,7 @@
       <c r="Q16" s="10"/>
     </row>
     <row r="17" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="117"/>
+      <c r="A17" s="120"/>
       <c r="B17" s="15">
         <v>2018</v>
       </c>
@@ -5564,7 +5567,7 @@
       <c r="Q17" s="10"/>
     </row>
     <row r="18" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="116" t="s">
+      <c r="A18" s="119" t="s">
         <v>19</v>
       </c>
       <c r="B18" s="9">
@@ -5615,7 +5618,7 @@
       <c r="Q18" s="10"/>
     </row>
     <row r="19" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="117"/>
+      <c r="A19" s="120"/>
       <c r="B19" s="15">
         <v>2018</v>
       </c>
@@ -5683,20 +5686,20 @@
       <c r="Q20" s="10"/>
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A21" s="132" t="s">
+      <c r="A21" s="118" t="s">
         <v>26</v>
       </c>
-      <c r="B21" s="132"/>
-      <c r="C21" s="132"/>
-      <c r="D21" s="132"/>
-      <c r="E21" s="132"/>
-      <c r="F21" s="132"/>
-      <c r="G21" s="132"/>
-      <c r="H21" s="132"/>
-      <c r="I21" s="132"/>
-      <c r="J21" s="132"/>
-      <c r="K21" s="132"/>
-      <c r="L21" s="132"/>
+      <c r="B21" s="118"/>
+      <c r="C21" s="118"/>
+      <c r="D21" s="118"/>
+      <c r="E21" s="118"/>
+      <c r="F21" s="118"/>
+      <c r="G21" s="118"/>
+      <c r="H21" s="118"/>
+      <c r="I21" s="118"/>
+      <c r="J21" s="118"/>
+      <c r="K21" s="118"/>
+      <c r="L21" s="118"/>
       <c r="M21" s="27"/>
       <c r="N21" s="20" t="s">
         <v>23</v>
@@ -5709,66 +5712,66 @@
       </c>
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A22" s="132" t="s">
+      <c r="A22" s="118" t="s">
         <v>20</v>
       </c>
-      <c r="B22" s="132"/>
-      <c r="C22" s="132"/>
-      <c r="D22" s="132"/>
-      <c r="E22" s="132"/>
-      <c r="F22" s="132"/>
-      <c r="G22" s="132"/>
-      <c r="H22" s="132"/>
-      <c r="I22" s="132"/>
-      <c r="J22" s="132"/>
-      <c r="K22" s="132"/>
-      <c r="L22" s="132"/>
-      <c r="M22" s="132"/>
-      <c r="N22" s="132"/>
-      <c r="O22" s="132"/>
-      <c r="P22" s="132"/>
+      <c r="B22" s="118"/>
+      <c r="C22" s="118"/>
+      <c r="D22" s="118"/>
+      <c r="E22" s="118"/>
+      <c r="F22" s="118"/>
+      <c r="G22" s="118"/>
+      <c r="H22" s="118"/>
+      <c r="I22" s="118"/>
+      <c r="J22" s="118"/>
+      <c r="K22" s="118"/>
+      <c r="L22" s="118"/>
+      <c r="M22" s="118"/>
+      <c r="N22" s="118"/>
+      <c r="O22" s="118"/>
+      <c r="P22" s="118"/>
       <c r="Q22" s="23"/>
       <c r="R22" s="24"/>
     </row>
     <row r="23" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A23" s="132" t="s">
+      <c r="A23" s="118" t="s">
         <v>27</v>
       </c>
-      <c r="B23" s="132"/>
-      <c r="C23" s="132"/>
-      <c r="D23" s="132"/>
-      <c r="E23" s="132"/>
-      <c r="F23" s="132"/>
-      <c r="G23" s="132"/>
-      <c r="H23" s="132"/>
-      <c r="I23" s="132"/>
-      <c r="J23" s="132"/>
-      <c r="K23" s="132"/>
-      <c r="L23" s="132"/>
-      <c r="M23" s="132"/>
-      <c r="N23" s="132"/>
+      <c r="B23" s="118"/>
+      <c r="C23" s="118"/>
+      <c r="D23" s="118"/>
+      <c r="E23" s="118"/>
+      <c r="F23" s="118"/>
+      <c r="G23" s="118"/>
+      <c r="H23" s="118"/>
+      <c r="I23" s="118"/>
+      <c r="J23" s="118"/>
+      <c r="K23" s="118"/>
+      <c r="L23" s="118"/>
+      <c r="M23" s="118"/>
+      <c r="N23" s="118"/>
       <c r="O23" s="30"/>
       <c r="P23" s="30"/>
       <c r="Q23" s="23"/>
       <c r="R23" s="24"/>
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A24" s="132" t="s">
+      <c r="A24" s="118" t="s">
         <v>28</v>
       </c>
-      <c r="B24" s="132"/>
-      <c r="C24" s="132"/>
-      <c r="D24" s="132"/>
-      <c r="E24" s="132"/>
-      <c r="F24" s="132"/>
-      <c r="G24" s="132"/>
-      <c r="H24" s="132"/>
-      <c r="I24" s="132"/>
-      <c r="J24" s="132"/>
-      <c r="K24" s="132"/>
-      <c r="L24" s="132"/>
-      <c r="M24" s="132"/>
-      <c r="N24" s="132"/>
+      <c r="B24" s="118"/>
+      <c r="C24" s="118"/>
+      <c r="D24" s="118"/>
+      <c r="E24" s="118"/>
+      <c r="F24" s="118"/>
+      <c r="G24" s="118"/>
+      <c r="H24" s="118"/>
+      <c r="I24" s="118"/>
+      <c r="J24" s="118"/>
+      <c r="K24" s="118"/>
+      <c r="L24" s="118"/>
+      <c r="M24" s="118"/>
+      <c r="N24" s="118"/>
       <c r="O24"/>
       <c r="P24"/>
     </row>
@@ -23162,14 +23165,6 @@
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="A23:N23"/>
-    <mergeCell ref="A24:N24"/>
-    <mergeCell ref="A12:A13"/>
-    <mergeCell ref="A14:A15"/>
-    <mergeCell ref="A16:A17"/>
-    <mergeCell ref="A18:A19"/>
-    <mergeCell ref="A21:L21"/>
-    <mergeCell ref="A22:P22"/>
     <mergeCell ref="A10:A11"/>
     <mergeCell ref="A1:P1"/>
     <mergeCell ref="A2:P2"/>
@@ -23186,6 +23181,14 @@
     <mergeCell ref="O4:P4"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="A8:A9"/>
+    <mergeCell ref="A23:N23"/>
+    <mergeCell ref="A24:N24"/>
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="A16:A17"/>
+    <mergeCell ref="A18:A19"/>
+    <mergeCell ref="A21:L21"/>
+    <mergeCell ref="A22:P22"/>
   </mergeCells>
   <conditionalFormatting sqref="H6">
     <cfRule type="expression" dxfId="158" priority="137">
@@ -23770,18 +23773,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:137" s="1" customFormat="1" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="133"/>
-      <c r="B1" s="133"/>
-      <c r="C1" s="133"/>
-      <c r="D1" s="133"/>
-      <c r="E1" s="133"/>
+      <c r="A1" s="135"/>
+      <c r="B1" s="135"/>
+      <c r="C1" s="135"/>
+      <c r="D1" s="135"/>
+      <c r="E1" s="135"/>
     </row>
     <row r="2" spans="1:137" s="1" customFormat="1" ht="22.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="118"/>
-      <c r="B2" s="118"/>
-      <c r="C2" s="118"/>
-      <c r="D2" s="118"/>
-      <c r="E2" s="118"/>
+      <c r="A2" s="122"/>
+      <c r="B2" s="122"/>
+      <c r="C2" s="122"/>
+      <c r="D2" s="122"/>
+      <c r="E2" s="122"/>
     </row>
     <row r="3" spans="1:137" x14ac:dyDescent="0.25">
       <c r="A3" s="2"/>
@@ -31633,7 +31636,7 @@
   <sheetPr codeName="Лист6">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:CJ932"/>
+  <dimension ref="A1:DA931"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="47" style="76" bestFit="1" customWidth="1"/>
@@ -31653,43 +31656,43 @@
     <col min="17" max="16384" width="9.140625" style="73"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:88" s="71" customFormat="1" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="135" t="s">
+    <row r="1" spans="1:105" s="71" customFormat="1" ht="21" x14ac:dyDescent="0.35">
+      <c r="A1" s="136" t="s">
         <v>63</v>
       </c>
-      <c r="B1" s="135"/>
-      <c r="C1" s="135"/>
-      <c r="D1" s="135"/>
-      <c r="E1" s="135"/>
-      <c r="F1" s="135"/>
-      <c r="G1" s="135"/>
-      <c r="H1" s="135"/>
-      <c r="I1" s="135"/>
-      <c r="J1" s="135"/>
-      <c r="K1" s="135"/>
-      <c r="L1" s="135"/>
-      <c r="M1" s="135"/>
-      <c r="N1" s="135"/>
-    </row>
-    <row r="2" spans="1:88" s="71" customFormat="1" ht="21" x14ac:dyDescent="0.35">
-      <c r="A2" s="136" t="s">
+      <c r="B1" s="136"/>
+      <c r="C1" s="136"/>
+      <c r="D1" s="136"/>
+      <c r="E1" s="136"/>
+      <c r="F1" s="136"/>
+      <c r="G1" s="136"/>
+      <c r="H1" s="136"/>
+      <c r="I1" s="136"/>
+      <c r="J1" s="136"/>
+      <c r="K1" s="136"/>
+      <c r="L1" s="136"/>
+      <c r="M1" s="136"/>
+      <c r="N1" s="136"/>
+    </row>
+    <row r="2" spans="1:105" s="71" customFormat="1" ht="21" x14ac:dyDescent="0.35">
+      <c r="A2" s="137" t="s">
         <v>70</v>
       </c>
-      <c r="B2" s="136"/>
-      <c r="C2" s="136"/>
-      <c r="D2" s="136"/>
-      <c r="E2" s="136"/>
-      <c r="F2" s="136"/>
-      <c r="G2" s="136"/>
-      <c r="H2" s="136"/>
-      <c r="I2" s="136"/>
-      <c r="J2" s="136"/>
-      <c r="K2" s="136"/>
-      <c r="L2" s="136"/>
-      <c r="M2" s="136"/>
-      <c r="N2" s="136"/>
-    </row>
-    <row r="3" spans="1:88" ht="9" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="137"/>
+      <c r="C2" s="137"/>
+      <c r="D2" s="137"/>
+      <c r="E2" s="137"/>
+      <c r="F2" s="137"/>
+      <c r="G2" s="137"/>
+      <c r="H2" s="137"/>
+      <c r="I2" s="137"/>
+      <c r="J2" s="137"/>
+      <c r="K2" s="137"/>
+      <c r="L2" s="137"/>
+      <c r="M2" s="137"/>
+      <c r="N2" s="137"/>
+    </row>
+    <row r="3" spans="1:105" ht="9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="104"/>
       <c r="B3" s="104"/>
       <c r="C3" s="104"/>
@@ -31705,45 +31708,45 @@
       <c r="M3" s="104"/>
       <c r="N3" s="104"/>
     </row>
-    <row r="4" spans="1:88" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="134" t="s">
+    <row r="4" spans="1:105" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="138" t="s">
         <v>38</v>
       </c>
-      <c r="B4" s="137" t="s">
+      <c r="B4" s="139" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="134" t="s">
+      <c r="C4" s="138" t="s">
         <v>36</v>
       </c>
-      <c r="D4" s="134"/>
-      <c r="E4" s="134" t="s">
+      <c r="D4" s="138"/>
+      <c r="E4" s="138" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="134"/>
-      <c r="G4" s="134" t="s">
+      <c r="F4" s="138"/>
+      <c r="G4" s="138" t="s">
         <v>7</v>
       </c>
-      <c r="H4" s="134"/>
-      <c r="I4" s="134" t="s">
+      <c r="H4" s="138"/>
+      <c r="I4" s="138" t="s">
         <v>8</v>
       </c>
-      <c r="J4" s="134"/>
-      <c r="K4" s="134" t="s">
+      <c r="J4" s="138"/>
+      <c r="K4" s="138" t="s">
         <v>37</v>
       </c>
-      <c r="L4" s="134"/>
-      <c r="M4" s="134" t="s">
+      <c r="L4" s="138"/>
+      <c r="M4" s="138" t="s">
         <v>9</v>
       </c>
-      <c r="N4" s="134"/>
-      <c r="O4" s="134" t="s">
+      <c r="N4" s="138"/>
+      <c r="O4" s="138" t="s">
         <v>44</v>
       </c>
-      <c r="P4" s="134"/>
-    </row>
-    <row r="5" spans="1:88" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="134"/>
-      <c r="B5" s="137"/>
+      <c r="P4" s="138"/>
+    </row>
+    <row r="5" spans="1:105" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="138"/>
+      <c r="B5" s="139"/>
       <c r="C5" s="114" t="s">
         <v>11</v>
       </c>
@@ -31787,12 +31790,12 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:88" s="77" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="141" t="s">
+    <row r="6" spans="1:105" s="77" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="117" t="s">
         <v>13</v>
       </c>
       <c r="B6" s="107">
-        <v>1438.9290139999998</v>
+        <v>1522.950726</v>
       </c>
       <c r="C6" s="108">
         <v>0</v>
@@ -31804,39 +31807,37 @@
         <v>2.39127</v>
       </c>
       <c r="F6" s="108">
-        <v>0.23991233431321221</v>
+        <v>0.20841670785337121</v>
       </c>
       <c r="G6" s="107">
-        <v>236.423564</v>
+        <v>259.90216400000003</v>
       </c>
       <c r="H6" s="107">
-        <v>23.720001976309295</v>
+        <v>22.652378604192329</v>
       </c>
       <c r="I6" s="107">
-        <v>660.70211999999992</v>
+        <v>779.23487499999999</v>
       </c>
       <c r="J6" s="107">
-        <v>66.287197972160413</v>
+        <v>67.91603093420369</v>
       </c>
       <c r="K6" s="107">
-        <f>I6+G6+E6+C6</f>
-        <v>899.51695399999983</v>
+        <v>1041.528309</v>
       </c>
       <c r="L6" s="107">
-        <f>F6+D6+H6+J6</f>
-        <v>90.247112282782922</v>
+        <v>90.776826246249385</v>
       </c>
       <c r="M6" s="107">
-        <v>97.049623999999994</v>
+        <v>105.66212400000001</v>
       </c>
       <c r="N6" s="107">
-        <v>9.736835170457347</v>
+        <v>9.2092285809944876</v>
       </c>
       <c r="O6" s="107">
         <v>0.16</v>
       </c>
       <c r="P6" s="115">
-        <v>1.6052546759719295E-2</v>
+        <v>1.3945172756125154E-2</v>
       </c>
       <c r="Q6" s="76"/>
       <c r="R6" s="76"/>
@@ -31910,13 +31911,30 @@
       <c r="CH6" s="76"/>
       <c r="CI6" s="76"/>
       <c r="CJ6" s="76"/>
-    </row>
-    <row r="7" spans="1:88" s="79" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="141" t="s">
+      <c r="CK6" s="76"/>
+      <c r="CL6" s="76"/>
+      <c r="CM6" s="76"/>
+      <c r="CN6" s="76"/>
+      <c r="CO6" s="76"/>
+      <c r="CP6" s="76"/>
+      <c r="CQ6" s="76"/>
+      <c r="CR6" s="76"/>
+      <c r="CS6" s="76"/>
+      <c r="CT6" s="76"/>
+      <c r="CU6" s="76"/>
+      <c r="CV6" s="76"/>
+      <c r="CW6" s="76"/>
+      <c r="CX6" s="76"/>
+      <c r="CY6" s="76"/>
+      <c r="CZ6" s="76"/>
+      <c r="DA6" s="76"/>
+    </row>
+    <row r="7" spans="1:105" s="79" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="117" t="s">
         <v>14</v>
       </c>
       <c r="B7" s="107">
-        <v>254.040719</v>
+        <v>299.43596900000006</v>
       </c>
       <c r="C7" s="109">
         <v>0</v>
@@ -31934,27 +31952,25 @@
         <v>49.392344000000008</v>
       </c>
       <c r="H7" s="107">
-        <v>19.442687847218703</v>
+        <v>16.495127210318547</v>
       </c>
       <c r="I7" s="107">
-        <v>178.83263099999999</v>
+        <v>223.58788099999998</v>
       </c>
       <c r="J7" s="107">
-        <v>70.395262501205565</v>
+        <v>74.669680381651133</v>
       </c>
       <c r="K7" s="107">
-        <f t="shared" ref="K7:K36" si="0">I7+G7+E7+C7</f>
-        <v>228.224975</v>
+        <v>272.98022500000002</v>
       </c>
       <c r="L7" s="107">
-        <f t="shared" ref="L7:L36" si="1">F7+D7+H7+J7</f>
-        <v>89.837950348424272</v>
+        <v>91.164807591969677</v>
       </c>
       <c r="M7" s="107">
-        <v>25.815744000000002</v>
+        <v>26.455744000000003</v>
       </c>
       <c r="N7" s="107">
-        <v>10.162049651575741</v>
+        <v>8.8351924080303146</v>
       </c>
       <c r="O7" s="107">
         <v>0</v>
@@ -32034,13 +32050,30 @@
       <c r="CH7" s="78"/>
       <c r="CI7" s="78"/>
       <c r="CJ7" s="78"/>
-    </row>
-    <row r="8" spans="1:88" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="140" t="s">
+      <c r="CK7" s="78"/>
+      <c r="CL7" s="78"/>
+      <c r="CM7" s="78"/>
+      <c r="CN7" s="78"/>
+      <c r="CO7" s="78"/>
+      <c r="CP7" s="78"/>
+      <c r="CQ7" s="78"/>
+      <c r="CR7" s="78"/>
+      <c r="CS7" s="78"/>
+      <c r="CT7" s="78"/>
+      <c r="CU7" s="78"/>
+      <c r="CV7" s="78"/>
+      <c r="CW7" s="78"/>
+      <c r="CX7" s="78"/>
+      <c r="CY7" s="78"/>
+      <c r="CZ7" s="78"/>
+      <c r="DA7" s="78"/>
+    </row>
+    <row r="8" spans="1:105" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="116" t="s">
         <v>15</v>
       </c>
       <c r="B8" s="110">
-        <v>136.6</v>
+        <v>169.62</v>
       </c>
       <c r="C8" s="111"/>
       <c r="D8" s="111"/>
@@ -32050,44 +32083,38 @@
         <v>4.79</v>
       </c>
       <c r="H8" s="110">
-        <v>3.5065885797950225</v>
+        <v>2.823959438745431</v>
       </c>
       <c r="I8" s="112">
-        <v>130.54</v>
+        <v>162.91999999999999</v>
       </c>
       <c r="J8" s="110">
-        <v>95.563689604685209</v>
+        <v>96.049994104468809</v>
       </c>
       <c r="K8" s="110">
-        <f t="shared" si="0"/>
-        <v>135.32999999999998</v>
+        <v>167.70999999999998</v>
       </c>
       <c r="L8" s="110">
-        <f t="shared" si="1"/>
-        <v>99.07027818448023</v>
+        <v>98.873953543214228</v>
       </c>
       <c r="M8" s="110">
-        <v>1.27</v>
+        <v>1.91</v>
       </c>
       <c r="N8" s="110">
-        <v>0.92972181551976585</v>
+        <v>1.1260464567857562</v>
       </c>
       <c r="O8" s="110"/>
       <c r="P8" s="110"/>
     </row>
-    <row r="9" spans="1:88" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="140" t="s">
+    <row r="9" spans="1:105" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="116" t="s">
         <v>17</v>
       </c>
       <c r="B9" s="110">
-        <v>101.87631500000001</v>
-      </c>
-      <c r="C9" s="111">
-        <v>0</v>
-      </c>
-      <c r="D9" s="111">
-        <v>0</v>
-      </c>
+        <v>114.251565</v>
+      </c>
+      <c r="C9" s="111"/>
+      <c r="D9" s="111"/>
       <c r="E9" s="111">
         <v>0</v>
       </c>
@@ -32098,27 +32125,25 @@
         <v>42.602804000000006</v>
       </c>
       <c r="H9" s="110">
-        <v>41.818163525054871</v>
+        <v>37.28859556540867</v>
       </c>
       <c r="I9" s="112">
-        <v>39.221270999999994</v>
+        <v>51.596520999999996</v>
       </c>
       <c r="J9" s="110">
-        <v>38.498910173576647</v>
+        <v>45.160450099742611</v>
       </c>
       <c r="K9" s="110">
-        <f t="shared" si="0"/>
-        <v>81.824074999999993</v>
+        <v>94.199325000000002</v>
       </c>
       <c r="L9" s="110">
-        <f t="shared" si="1"/>
-        <v>80.317073698631518</v>
+        <v>82.449045665151289</v>
       </c>
       <c r="M9" s="110">
         <v>20.052240000000001</v>
       </c>
       <c r="N9" s="110">
-        <v>19.682926301368482</v>
+        <v>17.550954334848718</v>
       </c>
       <c r="O9" s="110">
         <v>0</v>
@@ -32127,8 +32152,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:88" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="140" t="s">
+    <row r="10" spans="1:105" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="116" t="s">
         <v>57</v>
       </c>
       <c r="B10" s="110">
@@ -32151,11 +32176,9 @@
         <v>65.741904053742203</v>
       </c>
       <c r="K10" s="110">
-        <f t="shared" si="0"/>
         <v>3.97994</v>
       </c>
       <c r="L10" s="110">
-        <f t="shared" si="1"/>
         <v>92.770115451585156</v>
       </c>
       <c r="M10" s="110">
@@ -32167,8 +32190,8 @@
       <c r="O10" s="110"/>
       <c r="P10" s="110"/>
     </row>
-    <row r="11" spans="1:88" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="140" t="s">
+    <row r="11" spans="1:105" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="116" t="s">
         <v>45</v>
       </c>
       <c r="B11" s="110">
@@ -32191,11 +32214,9 @@
         <v>11.456483658347336</v>
       </c>
       <c r="K11" s="110">
-        <f t="shared" si="0"/>
         <v>1.48996</v>
       </c>
       <c r="L11" s="110">
-        <f t="shared" si="1"/>
         <v>26.262696768402975</v>
       </c>
       <c r="M11" s="110">
@@ -32207,8 +32228,8 @@
       <c r="O11" s="110"/>
       <c r="P11" s="110"/>
     </row>
-    <row r="12" spans="1:88" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="140" t="s">
+    <row r="12" spans="1:105" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="116" t="s">
         <v>16</v>
       </c>
       <c r="B12" s="110">
@@ -32239,11 +32260,9 @@
         <v>100</v>
       </c>
       <c r="K12" s="110">
-        <f t="shared" si="0"/>
         <v>5.601</v>
       </c>
       <c r="L12" s="110">
-        <f t="shared" si="1"/>
         <v>100</v>
       </c>
       <c r="M12" s="110">
@@ -32259,12 +32278,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:88" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="141" t="s">
+    <row r="13" spans="1:105" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="117" t="s">
         <v>46</v>
       </c>
       <c r="B13" s="107">
-        <v>695.08834000000002</v>
+        <v>708.90910200000008</v>
       </c>
       <c r="C13" s="109">
         <v>0</v>
@@ -32276,43 +32295,41 @@
         <v>2.39127</v>
       </c>
       <c r="F13" s="109">
-        <v>0.65284867745362507</v>
+        <v>0.54727400890736067</v>
       </c>
       <c r="G13" s="107">
-        <v>137.98782</v>
+        <v>161.46642</v>
       </c>
       <c r="H13" s="107">
-        <v>37.67251953635887</v>
+        <v>36.953742144266286</v>
       </c>
       <c r="I13" s="107">
-        <v>170.14359999999999</v>
+        <v>209.35207000000003</v>
       </c>
       <c r="J13" s="107">
-        <v>46.451477347684957</v>
+        <v>47.913011337889237</v>
       </c>
       <c r="K13" s="107">
-        <f t="shared" si="0"/>
-        <v>310.52269000000001</v>
+        <v>373.20976000000002</v>
       </c>
       <c r="L13" s="107">
-        <f t="shared" si="1"/>
-        <v>84.776845561497453</v>
+        <v>85.414027491062882</v>
       </c>
       <c r="M13" s="107">
-        <v>55.599739999999997</v>
+        <v>63.572240000000001</v>
       </c>
       <c r="N13" s="107">
-        <v>15.179472299558567</v>
+        <v>14.549354376553408</v>
       </c>
       <c r="O13" s="107">
         <v>0.16</v>
       </c>
       <c r="P13" s="115">
-        <v>4.3682138943983748E-2</v>
-      </c>
-    </row>
-    <row r="14" spans="1:88" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="140" t="s">
+        <v>3.6618132383703095E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:105" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="116" t="s">
         <v>48</v>
       </c>
       <c r="B14" s="110">
@@ -32325,30 +32342,28 @@
       <c r="G14" s="110"/>
       <c r="H14" s="110"/>
       <c r="I14" s="112">
-        <v>14.76295</v>
+        <v>30.347079999999998</v>
       </c>
       <c r="J14" s="110">
-        <v>41.688304390318841</v>
+        <v>55.91074938298808</v>
       </c>
       <c r="K14" s="110">
-        <f t="shared" si="0"/>
-        <v>14.76295</v>
+        <v>30.347079999999998</v>
       </c>
       <c r="L14" s="110">
-        <f t="shared" si="1"/>
-        <v>41.688304390318841</v>
+        <v>55.91074938298808</v>
       </c>
       <c r="M14" s="110">
-        <v>20.649740000000001</v>
+        <v>23.930640000000004</v>
       </c>
       <c r="N14" s="110">
-        <v>58.311695609681166</v>
+        <v>44.08925061701192</v>
       </c>
       <c r="O14" s="110"/>
       <c r="P14" s="110"/>
     </row>
-    <row r="15" spans="1:88" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="140" t="s">
+    <row r="15" spans="1:105" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="116" t="s">
         <v>58</v>
       </c>
       <c r="B15" s="110">
@@ -32371,11 +32386,9 @@
         <v>44.089456869009581</v>
       </c>
       <c r="K15" s="110">
-        <f t="shared" si="0"/>
         <v>12.52</v>
       </c>
       <c r="L15" s="110">
-        <f t="shared" si="1"/>
         <v>100</v>
       </c>
       <c r="M15" s="110"/>
@@ -32383,12 +32396,12 @@
       <c r="O15" s="110"/>
       <c r="P15" s="110"/>
     </row>
-    <row r="16" spans="1:88" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="140" t="s">
+    <row r="16" spans="1:105" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="116" t="s">
         <v>51</v>
       </c>
       <c r="B16" s="110">
-        <v>9.844339999999999</v>
+        <v>16.96294</v>
       </c>
       <c r="C16" s="111"/>
       <c r="D16" s="111"/>
@@ -32396,27 +32409,25 @@
         <v>2.39127</v>
       </c>
       <c r="F16" s="111">
-        <v>24.29081076029475</v>
+        <v>14.097025633528151</v>
       </c>
       <c r="G16" s="110">
-        <v>2.2898200000000002</v>
+        <v>9.4084199999999996</v>
       </c>
       <c r="H16" s="110">
-        <v>23.260269352744832</v>
+        <v>55.46455979918575</v>
       </c>
       <c r="I16" s="112">
         <v>5.1632499999999997</v>
       </c>
       <c r="J16" s="110">
-        <v>52.448919886960432</v>
+        <v>30.438414567286092</v>
       </c>
       <c r="K16" s="110">
-        <f t="shared" si="0"/>
-        <v>9.8443400000000008</v>
+        <v>16.96294</v>
       </c>
       <c r="L16" s="110">
-        <f t="shared" si="1"/>
-        <v>100.00000000000001</v>
+        <v>100</v>
       </c>
       <c r="M16" s="110"/>
       <c r="N16" s="110"/>
@@ -32424,47 +32435,45 @@
       <c r="P16" s="110"/>
     </row>
     <row r="17" spans="1:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="140" t="s">
+      <c r="A17" s="116" t="s">
         <v>64</v>
       </c>
       <c r="B17" s="110">
-        <v>78.221999999999994</v>
+        <v>81.414000000000001</v>
       </c>
       <c r="C17" s="111"/>
       <c r="D17" s="111"/>
       <c r="E17" s="111"/>
       <c r="F17" s="111"/>
       <c r="G17" s="110">
-        <v>14.417999999999999</v>
+        <v>19.518000000000001</v>
       </c>
       <c r="H17" s="110">
-        <v>40.335259921556343</v>
+        <v>46.098535324024191</v>
       </c>
       <c r="I17" s="112">
-        <v>10.997400000000001</v>
+        <v>12.49174</v>
       </c>
       <c r="J17" s="110">
-        <v>30.765916733341918</v>
+        <v>29.503582213778358</v>
       </c>
       <c r="K17" s="110">
-        <f t="shared" si="0"/>
-        <v>25.415399999999998</v>
+        <v>32.009740000000001</v>
       </c>
       <c r="L17" s="110">
-        <f t="shared" si="1"/>
-        <v>71.101176654898268</v>
+        <v>75.602117537802542</v>
       </c>
       <c r="M17" s="110">
         <v>10.33</v>
       </c>
       <c r="N17" s="110">
-        <v>28.89882334510175</v>
+        <v>24.397882462197455</v>
       </c>
       <c r="O17" s="110"/>
       <c r="P17" s="110"/>
     </row>
     <row r="18" spans="1:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="140" t="s">
+      <c r="A18" s="116" t="s">
         <v>47</v>
       </c>
       <c r="B18" s="110">
@@ -32475,40 +32484,38 @@
       <c r="E18" s="111"/>
       <c r="F18" s="111"/>
       <c r="G18" s="110">
-        <v>114.28</v>
+        <v>125.54</v>
       </c>
       <c r="H18" s="110">
-        <v>41.897638949992668</v>
+        <v>40.512456434748927</v>
       </c>
       <c r="I18" s="112">
-        <v>133.69999999999999</v>
+        <v>155.83000000000001</v>
       </c>
       <c r="J18" s="110">
-        <v>49.017451239184631</v>
+        <v>50.287207951465071</v>
       </c>
       <c r="K18" s="110">
-        <f t="shared" si="0"/>
-        <v>247.98</v>
+        <v>281.37</v>
       </c>
       <c r="L18" s="110">
-        <f t="shared" si="1"/>
-        <v>90.915090189177306</v>
+        <v>90.799664386214005</v>
       </c>
       <c r="M18" s="110">
-        <v>24.62</v>
+        <v>28.35</v>
       </c>
       <c r="N18" s="110">
-        <v>9.0262501833113369</v>
+        <v>9.1487027236349547</v>
       </c>
       <c r="O18" s="110">
         <v>0.16</v>
       </c>
       <c r="P18" s="110">
-        <v>5.865962751136531E-2</v>
+        <v>5.1632890151026199E-2</v>
       </c>
     </row>
     <row r="19" spans="1:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="141" t="s">
+      <c r="A19" s="117" t="s">
         <v>18</v>
       </c>
       <c r="B19" s="107">
@@ -32539,12 +32546,10 @@
         <v>71.393276507761399</v>
       </c>
       <c r="K19" s="107">
-        <f t="shared" si="0"/>
         <v>78.570754999999991</v>
       </c>
       <c r="L19" s="107">
-        <f t="shared" si="1"/>
-        <v>92.973993150851484</v>
+        <v>92.97399315085147</v>
       </c>
       <c r="M19" s="107">
         <v>5.9375599999999995</v>
@@ -32555,12 +32560,12 @@
       <c r="O19" s="107">
         <v>0</v>
       </c>
-      <c r="P19" s="107">
+      <c r="P19" s="115">
         <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="140" t="s">
+      <c r="A20" s="116" t="s">
         <v>59</v>
       </c>
       <c r="B20" s="110">
@@ -32579,11 +32584,9 @@
       <c r="I20" s="112"/>
       <c r="J20" s="110"/>
       <c r="K20" s="110">
-        <f t="shared" si="0"/>
         <v>0.31</v>
       </c>
       <c r="L20" s="110">
-        <f t="shared" si="1"/>
         <v>100</v>
       </c>
       <c r="M20" s="110"/>
@@ -32592,7 +32595,7 @@
       <c r="P20" s="110"/>
     </row>
     <row r="21" spans="1:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="140" t="s">
+      <c r="A21" s="116" t="s">
         <v>60</v>
       </c>
       <c r="B21" s="110">
@@ -32611,11 +32614,9 @@
         <v>100</v>
       </c>
       <c r="K21" s="110">
-        <f t="shared" si="0"/>
         <v>1.34</v>
       </c>
       <c r="L21" s="110">
-        <f t="shared" si="1"/>
         <v>100</v>
       </c>
       <c r="M21" s="110"/>
@@ -32624,7 +32625,7 @@
       <c r="P21" s="110"/>
     </row>
     <row r="22" spans="1:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="140" t="s">
+      <c r="A22" s="116" t="s">
         <v>19</v>
       </c>
       <c r="B22" s="110">
@@ -32647,12 +32648,10 @@
         <v>71.197748831846269</v>
       </c>
       <c r="K22" s="110">
-        <f t="shared" si="0"/>
         <v>76.920755</v>
       </c>
       <c r="L22" s="110">
-        <f t="shared" si="1"/>
-        <v>92.834080683393097</v>
+        <v>92.834080683393083</v>
       </c>
       <c r="M22" s="110">
         <v>5.9375599999999995</v>
@@ -32664,7 +32663,7 @@
       <c r="P22" s="110"/>
     </row>
     <row r="23" spans="1:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="141" t="s">
+      <c r="A23" s="117" t="s">
         <v>52</v>
       </c>
       <c r="B23" s="107">
@@ -32678,33 +32677,31 @@
         <v>0.21</v>
       </c>
       <c r="H23" s="107">
-        <v>0.5351234384524719</v>
+        <v>0.48325651932604952</v>
       </c>
       <c r="I23" s="107">
-        <v>35.629621999999998</v>
+        <v>39.841521999999998</v>
       </c>
       <c r="J23" s="107">
-        <v>90.791646835246851</v>
+        <v>91.68416783986774</v>
       </c>
       <c r="K23" s="107">
-        <f t="shared" si="0"/>
-        <v>35.839621999999999</v>
+        <v>40.051521999999999</v>
       </c>
       <c r="L23" s="107">
-        <f t="shared" si="1"/>
-        <v>91.326770273699324</v>
+        <v>92.167424359193788</v>
       </c>
       <c r="M23" s="107">
         <v>3.4036599999999999</v>
       </c>
       <c r="N23" s="107">
-        <v>8.6732297263006704</v>
+        <v>7.8325756408061986</v>
       </c>
       <c r="O23" s="107"/>
-      <c r="P23" s="107"/>
+      <c r="P23" s="115"/>
     </row>
     <row r="24" spans="1:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="140" t="s">
+      <c r="A24" s="116" t="s">
         <v>61</v>
       </c>
       <c r="B24" s="110">
@@ -32723,11 +32720,9 @@
         <v>100</v>
       </c>
       <c r="K24" s="110">
-        <f t="shared" si="0"/>
         <v>5.3969399999999998</v>
       </c>
       <c r="L24" s="110">
-        <f t="shared" si="1"/>
         <v>100</v>
       </c>
       <c r="M24" s="110"/>
@@ -32735,8 +32730,8 @@
       <c r="O24" s="110"/>
       <c r="P24" s="110"/>
     </row>
-    <row r="25" spans="1:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="140" t="s">
+    <row r="25" spans="1:16" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A25" s="116" t="s">
         <v>55</v>
       </c>
       <c r="B25" s="110">
@@ -32755,11 +32750,9 @@
         <v>100</v>
       </c>
       <c r="K25" s="110">
-        <f t="shared" si="0"/>
         <v>2.5619999999999998</v>
       </c>
       <c r="L25" s="110">
-        <f t="shared" si="1"/>
         <v>100</v>
       </c>
       <c r="M25" s="110"/>
@@ -32768,7 +32761,7 @@
       <c r="P25" s="110"/>
     </row>
     <row r="26" spans="1:16" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A26" s="140" t="s">
+      <c r="A26" s="116" t="s">
         <v>65</v>
       </c>
       <c r="B26" s="110">
@@ -32781,17 +32774,15 @@
       <c r="G26" s="110"/>
       <c r="H26" s="110"/>
       <c r="I26" s="112">
-        <v>0.46954000000000001</v>
+        <v>3.61632</v>
       </c>
       <c r="J26" s="110">
         <v>100</v>
       </c>
       <c r="K26" s="110">
-        <f t="shared" si="0"/>
-        <v>0.46954000000000001</v>
+        <v>3.61632</v>
       </c>
       <c r="L26" s="110">
-        <f t="shared" si="1"/>
         <v>100</v>
       </c>
       <c r="M26" s="110"/>
@@ -32800,7 +32791,7 @@
       <c r="P26" s="110"/>
     </row>
     <row r="27" spans="1:16" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A27" s="140" t="s">
+      <c r="A27" s="116" t="s">
         <v>68</v>
       </c>
       <c r="B27" s="110">
@@ -32813,30 +32804,28 @@
       <c r="G27" s="110"/>
       <c r="H27" s="110"/>
       <c r="I27" s="112">
-        <v>16.993942000000001</v>
+        <v>18.059062000000001</v>
       </c>
       <c r="J27" s="110">
-        <v>93.755531479379499</v>
+        <v>94.102107235910808</v>
       </c>
       <c r="K27" s="110">
-        <f t="shared" si="0"/>
-        <v>16.993942000000001</v>
+        <v>18.059062000000001</v>
       </c>
       <c r="L27" s="110">
-        <f t="shared" si="1"/>
-        <v>93.755531479379499</v>
+        <v>94.102107235910808</v>
       </c>
       <c r="M27" s="110">
         <v>1.1318600000000001</v>
       </c>
       <c r="N27" s="110">
-        <v>6.2444685206204946</v>
+        <v>5.8978927640891881</v>
       </c>
       <c r="O27" s="110"/>
       <c r="P27" s="110"/>
     </row>
     <row r="28" spans="1:16" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A28" s="140" t="s">
+      <c r="A28" s="116" t="s">
         <v>62</v>
       </c>
       <c r="B28" s="110">
@@ -32859,12 +32848,10 @@
         <v>79.169919006252883</v>
       </c>
       <c r="K28" s="110">
-        <f t="shared" si="0"/>
         <v>9.6427000000000014</v>
       </c>
       <c r="L28" s="110">
-        <f t="shared" si="1"/>
-        <v>80.93247723362289</v>
+        <v>80.932477233622905</v>
       </c>
       <c r="M28" s="110">
         <v>2.2717999999999998</v>
@@ -32876,7 +32863,7 @@
       <c r="P28" s="110"/>
     </row>
     <row r="29" spans="1:16" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A29" s="140" t="s">
+      <c r="A29" s="116" t="s">
         <v>67</v>
       </c>
       <c r="B29" s="110">
@@ -32895,11 +32882,9 @@
         <v>100</v>
       </c>
       <c r="K29" s="110">
-        <f t="shared" si="0"/>
         <v>0.77449999999999997</v>
       </c>
       <c r="L29" s="110">
-        <f t="shared" si="1"/>
         <v>100</v>
       </c>
       <c r="M29" s="110"/>
@@ -32908,11 +32893,11 @@
       <c r="P29" s="110"/>
     </row>
     <row r="30" spans="1:16" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A30" s="141" t="s">
+      <c r="A30" s="117" t="s">
         <v>49</v>
       </c>
       <c r="B30" s="107">
-        <v>269.95399999999995</v>
+        <v>279.89600000000002</v>
       </c>
       <c r="C30" s="109">
         <v>0</v>
@@ -32930,41 +32915,39 @@
         <v>0.61799999999999999</v>
       </c>
       <c r="H30" s="107">
-        <v>0.33400597163763968</v>
+        <v>0.30182963409940711</v>
       </c>
       <c r="I30" s="107">
-        <v>183.624312</v>
+        <v>203.34894699999998</v>
       </c>
       <c r="J30" s="107">
-        <v>99.242098294260686</v>
+        <v>99.315110465226084</v>
       </c>
       <c r="K30" s="107">
-        <f t="shared" si="0"/>
-        <v>184.242312</v>
+        <v>203.96694699999998</v>
       </c>
       <c r="L30" s="107">
-        <f t="shared" si="1"/>
-        <v>99.576104265898323</v>
+        <v>99.61694009932549</v>
       </c>
       <c r="M30" s="107">
         <v>0.78432000000000002</v>
       </c>
       <c r="N30" s="107">
-        <v>0.42389573410167242</v>
+        <v>0.38305990067450968</v>
       </c>
       <c r="O30" s="107">
         <v>0</v>
       </c>
-      <c r="P30" s="107">
+      <c r="P30" s="115">
         <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:16" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A31" s="140" t="s">
+      <c r="A31" s="116" t="s">
         <v>66</v>
       </c>
       <c r="B31" s="110">
-        <v>10.9</v>
+        <v>15.189</v>
       </c>
       <c r="C31" s="111"/>
       <c r="D31" s="111"/>
@@ -32979,11 +32962,9 @@
         <v>96.815291618343096</v>
       </c>
       <c r="K31" s="110">
-        <f t="shared" si="0"/>
         <v>8.6433420000000005</v>
       </c>
       <c r="L31" s="110">
-        <f t="shared" si="1"/>
         <v>96.815291618343096</v>
       </c>
       <c r="M31" s="110">
@@ -32996,7 +32977,7 @@
       <c r="P31" s="110"/>
     </row>
     <row r="32" spans="1:16" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A32" s="140" t="s">
+      <c r="A32" s="116" t="s">
         <v>69</v>
       </c>
       <c r="B32" s="110">
@@ -33015,11 +32996,9 @@
       <c r="I32" s="112"/>
       <c r="J32" s="110"/>
       <c r="K32" s="110">
-        <f t="shared" si="0"/>
         <v>0.61799999999999999</v>
       </c>
       <c r="L32" s="110">
-        <f t="shared" si="1"/>
         <v>100</v>
       </c>
       <c r="M32" s="110"/>
@@ -33028,11 +33007,11 @@
       <c r="P32" s="110"/>
     </row>
     <row r="33" spans="1:16" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A33" s="140" t="s">
+      <c r="A33" s="116" t="s">
         <v>50</v>
       </c>
       <c r="B33" s="110">
-        <v>258.43599999999998</v>
+        <v>264.089</v>
       </c>
       <c r="C33" s="111"/>
       <c r="D33" s="111"/>
@@ -33041,34 +33020,32 @@
       <c r="G33" s="110"/>
       <c r="H33" s="110"/>
       <c r="I33" s="112">
-        <v>174.98097000000001</v>
+        <v>194.70560499999999</v>
       </c>
       <c r="J33" s="110">
-        <v>99.715068819143184</v>
+        <v>99.743859813861391</v>
       </c>
       <c r="K33" s="110">
-        <f t="shared" si="0"/>
-        <v>174.98097000000001</v>
+        <v>194.70560499999999</v>
       </c>
       <c r="L33" s="110">
-        <f t="shared" si="1"/>
-        <v>99.715068819143184</v>
+        <v>99.743859813861391</v>
       </c>
       <c r="M33" s="110">
         <v>0.5</v>
       </c>
       <c r="N33" s="110">
-        <v>0.28493118085681884</v>
+        <v>0.25614018613861012</v>
       </c>
       <c r="O33" s="110"/>
       <c r="P33" s="110"/>
     </row>
     <row r="34" spans="1:16" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A34" s="141" t="s">
+      <c r="A34" s="117" t="s">
         <v>53</v>
       </c>
       <c r="B34" s="107">
-        <v>76.390199999999993</v>
+        <v>91.253900000000002</v>
       </c>
       <c r="C34" s="109">
         <v>0</v>
@@ -33086,41 +33063,39 @@
         <v>29.977900000000002</v>
       </c>
       <c r="H34" s="107">
-        <v>44.329480726119854</v>
+        <v>38.306645863601922</v>
       </c>
       <c r="I34" s="107">
-        <v>32.1387</v>
+        <v>42.7712</v>
       </c>
       <c r="J34" s="107">
-        <v>47.524739298368068</v>
+        <v>54.654302388135612</v>
       </c>
       <c r="K34" s="107">
-        <f t="shared" si="0"/>
-        <v>62.116600000000005</v>
+        <v>72.749099999999999</v>
       </c>
       <c r="L34" s="107">
-        <f t="shared" si="1"/>
-        <v>91.854220024487915</v>
+        <v>92.960948251737534</v>
       </c>
       <c r="M34" s="107">
         <v>5.5086000000000004</v>
       </c>
       <c r="N34" s="107">
-        <v>8.1457799755120899</v>
+        <v>7.0390517482624722</v>
       </c>
       <c r="O34" s="107">
         <v>0</v>
       </c>
-      <c r="P34" s="107">
+      <c r="P34" s="115">
         <v>0</v>
       </c>
     </row>
     <row r="35" spans="1:16" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A35" s="140" t="s">
+      <c r="A35" s="116" t="s">
         <v>56</v>
       </c>
       <c r="B35" s="110">
-        <v>26.985199999999999</v>
+        <v>41.8489</v>
       </c>
       <c r="C35" s="111">
         <v>0</v>
@@ -33138,27 +33113,25 @@
         <v>3.1278999999999999</v>
       </c>
       <c r="H35" s="110">
-        <v>12.037236580822929</v>
+        <v>8.9630548718110354</v>
       </c>
       <c r="I35" s="112">
-        <v>21.4587</v>
+        <v>30.371200000000002</v>
       </c>
       <c r="J35" s="110">
-        <v>82.580468882286837</v>
+        <v>87.029231152769384</v>
       </c>
       <c r="K35" s="110">
-        <f t="shared" si="0"/>
-        <v>24.586600000000001</v>
+        <v>33.499099999999999</v>
       </c>
       <c r="L35" s="110">
-        <f t="shared" si="1"/>
-        <v>94.617705463109772</v>
+        <v>95.992286024580409</v>
       </c>
       <c r="M35" s="110">
         <v>1.3986000000000001</v>
       </c>
       <c r="N35" s="110">
-        <v>5.38229453689023</v>
+        <v>4.0077139754195832</v>
       </c>
       <c r="O35" s="110">
         <v>0</v>
@@ -33168,7 +33141,7 @@
       </c>
     </row>
     <row r="36" spans="1:16" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A36" s="140" t="s">
+      <c r="A36" s="116" t="s">
         <v>54</v>
       </c>
       <c r="B36" s="110">
@@ -33190,27 +33163,25 @@
         <v>26.85</v>
       </c>
       <c r="H36" s="110">
-        <v>64.481268011527391</v>
+        <v>61.923431734317361</v>
       </c>
       <c r="I36" s="112">
-        <v>10.68</v>
+        <v>12.4</v>
       </c>
       <c r="J36" s="110">
-        <v>25.648414985590783</v>
+        <v>28.597785977859786</v>
       </c>
       <c r="K36" s="110">
-        <f t="shared" si="0"/>
-        <v>37.53</v>
+        <v>39.25</v>
       </c>
       <c r="L36" s="110">
-        <f t="shared" si="1"/>
-        <v>90.129682997118181</v>
+        <v>90.521217712177133</v>
       </c>
       <c r="M36" s="110">
         <v>4.1100000000000003</v>
       </c>
       <c r="N36" s="110">
-        <v>9.8703170028818477</v>
+        <v>9.4787822878228809</v>
       </c>
       <c r="O36" s="110">
         <v>0</v>
@@ -33219,21 +33190,35 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A37"/>
-      <c r="B37"/>
-      <c r="C37"/>
-      <c r="D37"/>
-      <c r="E37"/>
-      <c r="F37"/>
-      <c r="G37"/>
-      <c r="H37"/>
-      <c r="I37"/>
-      <c r="J37"/>
-      <c r="K37"/>
-      <c r="L37"/>
-      <c r="M37"/>
-      <c r="N37"/>
+    <row r="37" spans="1:16" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A37" s="116" t="s">
+        <v>71</v>
+      </c>
+      <c r="B37" s="110">
+        <v>3.5101619999999998</v>
+      </c>
+      <c r="C37" s="111"/>
+      <c r="D37" s="111"/>
+      <c r="E37" s="111"/>
+      <c r="F37" s="111"/>
+      <c r="G37" s="110"/>
+      <c r="H37" s="110"/>
+      <c r="I37" s="112"/>
+      <c r="J37" s="110"/>
+      <c r="K37" s="110">
+        <v>0</v>
+      </c>
+      <c r="L37" s="110">
+        <v>0</v>
+      </c>
+      <c r="M37" s="110">
+        <v>0.96160000000000001</v>
+      </c>
+      <c r="N37" s="110">
+        <v>100</v>
+      </c>
+      <c r="O37" s="110"/>
+      <c r="P37" s="110"/>
     </row>
     <row r="38" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A38"/>
@@ -47508,20 +47493,20 @@
       <c r="N929"/>
     </row>
     <row r="930" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A930"/>
-      <c r="B930"/>
-      <c r="C930"/>
-      <c r="D930"/>
-      <c r="E930"/>
-      <c r="F930"/>
-      <c r="G930"/>
-      <c r="H930"/>
-      <c r="I930"/>
-      <c r="J930"/>
-      <c r="K930"/>
-      <c r="L930"/>
-      <c r="M930"/>
-      <c r="N930"/>
+      <c r="A930" s="81"/>
+      <c r="B930" s="81"/>
+      <c r="C930" s="81"/>
+      <c r="D930" s="81"/>
+      <c r="E930" s="81"/>
+      <c r="F930" s="81"/>
+      <c r="G930" s="81"/>
+      <c r="H930" s="81"/>
+      <c r="I930" s="81"/>
+      <c r="J930" s="81"/>
+      <c r="K930" s="81"/>
+      <c r="L930" s="81"/>
+      <c r="M930" s="81"/>
+      <c r="N930" s="81"/>
     </row>
     <row r="931" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A931" s="81"/>
@@ -47539,25 +47524,12 @@
       <c r="M931" s="81"/>
       <c r="N931" s="81"/>
     </row>
-    <row r="932" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A932" s="81"/>
-      <c r="B932" s="81"/>
-      <c r="C932" s="81"/>
-      <c r="D932" s="81"/>
-      <c r="E932" s="81"/>
-      <c r="F932" s="81"/>
-      <c r="G932" s="81"/>
-      <c r="H932" s="81"/>
-      <c r="I932" s="81"/>
-      <c r="J932" s="81"/>
-      <c r="K932" s="81"/>
-      <c r="L932" s="81"/>
-      <c r="M932" s="81"/>
-      <c r="N932" s="81"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A5:CJ36" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
+  <autoFilter ref="A5:DA37" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
   <mergeCells count="11">
+    <mergeCell ref="O4:P4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="K4:L4"/>
     <mergeCell ref="A1:N1"/>
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A4:A5"/>
@@ -47566,9 +47538,6 @@
     <mergeCell ref="E4:F4"/>
     <mergeCell ref="G4:H4"/>
     <mergeCell ref="I4:J4"/>
-    <mergeCell ref="O4:P4"/>
-    <mergeCell ref="M4:N4"/>
-    <mergeCell ref="K4:L4"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.19685039370078741" bottom="0.19685039370078741" header="0" footer="0"/>
@@ -47602,39 +47571,39 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:122" s="71" customFormat="1" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="138" t="s">
+      <c r="A1" s="140" t="s">
         <v>42</v>
       </c>
-      <c r="B1" s="138"/>
-      <c r="C1" s="138"/>
-      <c r="D1" s="138"/>
-      <c r="E1" s="138"/>
-      <c r="F1" s="138"/>
-      <c r="G1" s="138"/>
-      <c r="H1" s="138"/>
-      <c r="I1" s="138"/>
-      <c r="J1" s="138"/>
-      <c r="K1" s="138"/>
-      <c r="L1" s="138"/>
-      <c r="M1" s="138"/>
+      <c r="B1" s="140"/>
+      <c r="C1" s="140"/>
+      <c r="D1" s="140"/>
+      <c r="E1" s="140"/>
+      <c r="F1" s="140"/>
+      <c r="G1" s="140"/>
+      <c r="H1" s="140"/>
+      <c r="I1" s="140"/>
+      <c r="J1" s="140"/>
+      <c r="K1" s="140"/>
+      <c r="L1" s="140"/>
+      <c r="M1" s="140"/>
     </row>
     <row r="2" spans="1:122" s="71" customFormat="1" ht="22.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="139" t="str">
-        <f>'Пшеница твердая 28 сен'!A2:N2</f>
-        <v>по состоянию на 28 сентября</v>
-      </c>
-      <c r="B2" s="139"/>
-      <c r="C2" s="139"/>
-      <c r="D2" s="139"/>
-      <c r="E2" s="139"/>
-      <c r="F2" s="139"/>
-      <c r="G2" s="139"/>
-      <c r="H2" s="139"/>
-      <c r="I2" s="139"/>
-      <c r="J2" s="139"/>
-      <c r="K2" s="139"/>
-      <c r="L2" s="139"/>
-      <c r="M2" s="139"/>
+      <c r="A2" s="141" t="str">
+        <f>'Пшеница твердая 5 окт'!A2:N2</f>
+        <v>по состоянию на 5 октября</v>
+      </c>
+      <c r="B2" s="141"/>
+      <c r="C2" s="141"/>
+      <c r="D2" s="141"/>
+      <c r="E2" s="141"/>
+      <c r="F2" s="141"/>
+      <c r="G2" s="141"/>
+      <c r="H2" s="141"/>
+      <c r="I2" s="141"/>
+      <c r="J2" s="141"/>
+      <c r="K2" s="141"/>
+      <c r="L2" s="141"/>
+      <c r="M2" s="141"/>
     </row>
     <row r="3" spans="1:122" x14ac:dyDescent="0.25">
       <c r="A3" s="72"/>
@@ -47652,36 +47621,36 @@
       <c r="M3" s="72"/>
     </row>
     <row r="4" spans="1:122" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="128" t="s">
+      <c r="A4" s="132" t="s">
         <v>38</v>
       </c>
-      <c r="B4" s="128" t="s">
+      <c r="B4" s="132" t="s">
         <v>36</v>
       </c>
-      <c r="C4" s="128"/>
-      <c r="D4" s="128" t="s">
+      <c r="C4" s="132"/>
+      <c r="D4" s="132" t="s">
         <v>6</v>
       </c>
-      <c r="E4" s="128"/>
-      <c r="F4" s="128" t="s">
+      <c r="E4" s="132"/>
+      <c r="F4" s="132" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="128"/>
-      <c r="H4" s="128" t="s">
+      <c r="G4" s="132"/>
+      <c r="H4" s="132" t="s">
         <v>8</v>
       </c>
-      <c r="I4" s="128"/>
-      <c r="J4" s="128" t="s">
+      <c r="I4" s="132"/>
+      <c r="J4" s="132" t="s">
         <v>37</v>
       </c>
-      <c r="K4" s="128"/>
-      <c r="L4" s="128" t="s">
+      <c r="K4" s="132"/>
+      <c r="L4" s="132" t="s">
         <v>9</v>
       </c>
-      <c r="M4" s="128"/>
+      <c r="M4" s="132"/>
     </row>
     <row r="5" spans="1:122" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="128"/>
+      <c r="A5" s="132"/>
       <c r="B5" s="90" t="s">
         <v>43</v>
       </c>
@@ -47721,56 +47690,56 @@
     </row>
     <row r="6" spans="1:122" s="77" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="94" t="str">
-        <f>'Пшеница твердая 28 сен'!A6</f>
+        <f>'Пшеница твердая 5 окт'!A6</f>
         <v>Всего</v>
       </c>
       <c r="B6" s="91" t="str">
-        <f>IF('Пшеница твердая 28 сен'!D6=0,"",'Пшеница твердая 28 сен'!D6-'Пшеница твердая 28 сен'!#REF!)</f>
+        <f>IF('Пшеница твердая 5 окт'!D6=0,"",'Пшеница твердая 5 окт'!D6-'Пшеница твердая 5 окт'!#REF!)</f>
         <v/>
       </c>
       <c r="C6" s="92">
-        <f>'Пшеница твердая 28 сен'!D6</f>
+        <f>'Пшеница твердая 5 окт'!D6</f>
         <v>0</v>
       </c>
       <c r="D6" s="97" t="e">
-        <f>IF('Пшеница твердая 28 сен'!F6=0,"",'Пшеница твердая 28 сен'!F6-'Пшеница твердая 28 сен'!#REF!)</f>
+        <f>IF('Пшеница твердая 5 окт'!F6=0,"",'Пшеница твердая 5 окт'!F6-'Пшеница твердая 5 окт'!#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="E6" s="92">
-        <f>'Пшеница твердая 28 сен'!F6</f>
-        <v>0.23991233431321221</v>
+        <f>'Пшеница твердая 5 окт'!F6</f>
+        <v>0.20841670785337121</v>
       </c>
       <c r="F6" s="97" t="e">
-        <f>IF('Пшеница твердая 28 сен'!H6=0,"",'Пшеница твердая 28 сен'!H6-'Пшеница твердая 28 сен'!#REF!)</f>
+        <f>IF('Пшеница твердая 5 окт'!H6=0,"",'Пшеница твердая 5 окт'!H6-'Пшеница твердая 5 окт'!#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="G6" s="92">
-        <f>'Пшеница твердая 28 сен'!H6</f>
-        <v>23.720001976309295</v>
+        <f>'Пшеница твердая 5 окт'!H6</f>
+        <v>22.652378604192329</v>
       </c>
       <c r="H6" s="97" t="e">
-        <f>IF('Пшеница твердая 28 сен'!J6=0,"",'Пшеница твердая 28 сен'!J6-'Пшеница твердая 28 сен'!#REF!)</f>
+        <f>IF('Пшеница твердая 5 окт'!J6=0,"",'Пшеница твердая 5 окт'!J6-'Пшеница твердая 5 окт'!#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="I6" s="92">
-        <f>'Пшеница твердая 28 сен'!J6</f>
-        <v>66.287197972160413</v>
+        <f>'Пшеница твердая 5 окт'!J6</f>
+        <v>67.91603093420369</v>
       </c>
       <c r="J6" s="97" t="e">
-        <f>IF('Пшеница твердая 28 сен'!L6=0,"",'Пшеница твердая 28 сен'!L6-'Пшеница твердая 28 сен'!#REF!)</f>
+        <f>IF('Пшеница твердая 5 окт'!L6=0,"",'Пшеница твердая 5 окт'!L6-'Пшеница твердая 5 окт'!#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="K6" s="92">
-        <f>'Пшеница твердая 28 сен'!L6</f>
-        <v>90.247112282782922</v>
+        <f>'Пшеница твердая 5 окт'!L6</f>
+        <v>90.776826246249385</v>
       </c>
       <c r="L6" s="99" t="e">
-        <f>IF('Пшеница твердая 28 сен'!N6=0,"",'Пшеница твердая 28 сен'!N6-'Пшеница твердая 28 сен'!#REF!)</f>
+        <f>IF('Пшеница твердая 5 окт'!N6=0,"",'Пшеница твердая 5 окт'!N6-'Пшеница твердая 5 окт'!#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="M6" s="92">
-        <f>'Пшеница твердая 28 сен'!N6</f>
-        <v>9.736835170457347</v>
+        <f>'Пшеница твердая 5 окт'!N6</f>
+        <v>9.2092285809944876</v>
       </c>
       <c r="N6" s="73"/>
       <c r="O6" s="73"/>
@@ -47884,56 +47853,56 @@
     </row>
     <row r="7" spans="1:122" s="79" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="95" t="str">
-        <f>'Пшеница твердая 28 сен'!A7</f>
+        <f>'Пшеница твердая 5 окт'!A7</f>
         <v>Южный фед. округ</v>
       </c>
       <c r="B7" s="101" t="str">
-        <f>IF('Пшеница твердая 28 сен'!D7=0,"",'Пшеница твердая 28 сен'!D7-'Пшеница твердая 28 сен'!#REF!)</f>
+        <f>IF('Пшеница твердая 5 окт'!D7=0,"",'Пшеница твердая 5 окт'!D7-'Пшеница твердая 5 окт'!#REF!)</f>
         <v/>
       </c>
       <c r="C7" s="93">
-        <f>'Пшеница твердая 28 сен'!D7</f>
+        <f>'Пшеница твердая 5 окт'!D7</f>
         <v>0</v>
       </c>
       <c r="D7" s="98" t="str">
-        <f>IF('Пшеница твердая 28 сен'!F7=0,"",'Пшеница твердая 28 сен'!F7-'Пшеница твердая 28 сен'!#REF!)</f>
+        <f>IF('Пшеница твердая 5 окт'!F7=0,"",'Пшеница твердая 5 окт'!F7-'Пшеница твердая 5 окт'!#REF!)</f>
         <v/>
       </c>
       <c r="E7" s="93">
-        <f>'Пшеница твердая 28 сен'!F7</f>
+        <f>'Пшеница твердая 5 окт'!F7</f>
         <v>0</v>
       </c>
       <c r="F7" s="98" t="e">
-        <f>IF('Пшеница твердая 28 сен'!H7=0,"",'Пшеница твердая 28 сен'!H7-'Пшеница твердая 28 сен'!#REF!)</f>
+        <f>IF('Пшеница твердая 5 окт'!H7=0,"",'Пшеница твердая 5 окт'!H7-'Пшеница твердая 5 окт'!#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="G7" s="93">
-        <f>'Пшеница твердая 28 сен'!H7</f>
-        <v>19.442687847218703</v>
+        <f>'Пшеница твердая 5 окт'!H7</f>
+        <v>16.495127210318547</v>
       </c>
       <c r="H7" s="98" t="e">
-        <f>IF('Пшеница твердая 28 сен'!J7=0,"",'Пшеница твердая 28 сен'!J7-'Пшеница твердая 28 сен'!#REF!)</f>
+        <f>IF('Пшеница твердая 5 окт'!J7=0,"",'Пшеница твердая 5 окт'!J7-'Пшеница твердая 5 окт'!#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="I7" s="93">
-        <f>'Пшеница твердая 28 сен'!J7</f>
-        <v>70.395262501205565</v>
+        <f>'Пшеница твердая 5 окт'!J7</f>
+        <v>74.669680381651133</v>
       </c>
       <c r="J7" s="98" t="e">
-        <f>IF('Пшеница твердая 28 сен'!L7=0,"",'Пшеница твердая 28 сен'!L7-'Пшеница твердая 28 сен'!#REF!)</f>
+        <f>IF('Пшеница твердая 5 окт'!L7=0,"",'Пшеница твердая 5 окт'!L7-'Пшеница твердая 5 окт'!#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="K7" s="93">
-        <f>'Пшеница твердая 28 сен'!L7</f>
-        <v>89.837950348424272</v>
+        <f>'Пшеница твердая 5 окт'!L7</f>
+        <v>91.164807591969677</v>
       </c>
       <c r="L7" s="100" t="e">
-        <f>IF('Пшеница твердая 28 сен'!N7=0,"",'Пшеница твердая 28 сен'!N7-'Пшеница твердая 28 сен'!#REF!)</f>
+        <f>IF('Пшеница твердая 5 окт'!N7=0,"",'Пшеница твердая 5 окт'!N7-'Пшеница твердая 5 окт'!#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="M7" s="93">
-        <f>'Пшеница твердая 28 сен'!N7</f>
-        <v>10.162049651575741</v>
+        <f>'Пшеница твердая 5 окт'!N7</f>
+        <v>8.8351924080303146</v>
       </c>
       <c r="N7" s="73"/>
       <c r="O7" s="73"/>
@@ -48047,55 +48016,55 @@
     </row>
     <row r="8" spans="1:122" s="77" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="96" t="e">
-        <f>'Пшеница твердая 28 сен'!#REF!</f>
+        <f>'Пшеница твердая 5 окт'!#REF!</f>
         <v>#REF!</v>
       </c>
       <c r="B8" s="91" t="e">
-        <f>IF('Пшеница твердая 28 сен'!#REF!=0,"",'Пшеница твердая 28 сен'!#REF!-'Пшеница твердая 28 сен'!#REF!)</f>
+        <f>IF('Пшеница твердая 5 окт'!#REF!=0,"",'Пшеница твердая 5 окт'!#REF!-'Пшеница твердая 5 окт'!#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="C8" s="92" t="e">
-        <f>'Пшеница твердая 28 сен'!#REF!</f>
+        <f>'Пшеница твердая 5 окт'!#REF!</f>
         <v>#REF!</v>
       </c>
       <c r="D8" s="91" t="e">
-        <f>IF('Пшеница твердая 28 сен'!#REF!=0,"",'Пшеница твердая 28 сен'!#REF!-'Пшеница твердая 28 сен'!#REF!)</f>
+        <f>IF('Пшеница твердая 5 окт'!#REF!=0,"",'Пшеница твердая 5 окт'!#REF!-'Пшеница твердая 5 окт'!#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="E8" s="92" t="e">
-        <f>'Пшеница твердая 28 сен'!#REF!</f>
+        <f>'Пшеница твердая 5 окт'!#REF!</f>
         <v>#REF!</v>
       </c>
       <c r="F8" s="91" t="e">
-        <f>IF('Пшеница твердая 28 сен'!#REF!=0,"",'Пшеница твердая 28 сен'!#REF!-'Пшеница твердая 28 сен'!#REF!)</f>
+        <f>IF('Пшеница твердая 5 окт'!#REF!=0,"",'Пшеница твердая 5 окт'!#REF!-'Пшеница твердая 5 окт'!#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="G8" s="92" t="e">
-        <f>'Пшеница твердая 28 сен'!#REF!</f>
+        <f>'Пшеница твердая 5 окт'!#REF!</f>
         <v>#REF!</v>
       </c>
       <c r="H8" s="91" t="e">
-        <f>IF('Пшеница твердая 28 сен'!#REF!=0,"",'Пшеница твердая 28 сен'!#REF!-'Пшеница твердая 28 сен'!#REF!)</f>
+        <f>IF('Пшеница твердая 5 окт'!#REF!=0,"",'Пшеница твердая 5 окт'!#REF!-'Пшеница твердая 5 окт'!#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="I8" s="92" t="e">
-        <f>'Пшеница твердая 28 сен'!#REF!</f>
+        <f>'Пшеница твердая 5 окт'!#REF!</f>
         <v>#REF!</v>
       </c>
       <c r="J8" s="91" t="e">
-        <f>IF('Пшеница твердая 28 сен'!#REF!=0,"",'Пшеница твердая 28 сен'!#REF!-'Пшеница твердая 28 сен'!#REF!)</f>
+        <f>IF('Пшеница твердая 5 окт'!#REF!=0,"",'Пшеница твердая 5 окт'!#REF!-'Пшеница твердая 5 окт'!#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="K8" s="92" t="e">
-        <f>'Пшеница твердая 28 сен'!#REF!</f>
+        <f>'Пшеница твердая 5 окт'!#REF!</f>
         <v>#REF!</v>
       </c>
       <c r="L8" s="91" t="e">
-        <f>IF('Пшеница твердая 28 сен'!#REF!=0,"",'Пшеница твердая 28 сен'!#REF!-'Пшеница твердая 28 сен'!#REF!)</f>
+        <f>IF('Пшеница твердая 5 окт'!#REF!=0,"",'Пшеница твердая 5 окт'!#REF!-'Пшеница твердая 5 окт'!#REF!)</f>
         <v>#REF!</v>
       </c>
       <c r="M8" s="92" t="e">
-        <f>'Пшеница твердая 28 сен'!#REF!</f>
+        <f>'Пшеница твердая 5 окт'!#REF!</f>
         <v>#REF!</v>
       </c>
       <c r="N8" s="73"/>

</xml_diff>